<commit_message>
Fix BLOCKING/RFC PROGRESS headers (CPP-1/EACOP/REMARK EACOP/REMARK CPP-EIT/REMARK CPP-1) + red BLOCK-point ITR rows
</commit_message>
<xml_diff>
--- a/EXCEL/1 - DASHBOARD.xlsx
+++ b/EXCEL/1 - DASHBOARD.xlsx
@@ -65,7 +65,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FFed7d31"/>
+      <color rgb="FF2e7d32"/>
       <sz val="10"/>
     </font>
     <font>
@@ -77,7 +77,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FFc00000"/>
+      <color rgb="FFed7d31"/>
       <sz val="10"/>
     </font>
     <font>
@@ -94,7 +94,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FF2e7d32"/>
+      <color rgb="FFc00000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -170,7 +170,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="37">
+  <fills count="38">
     <fill>
       <patternFill/>
     </fill>
@@ -239,6 +239,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFffeb9c"/>
+        <bgColor rgb="FFffeb9c"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFe8d5c4"/>
         <bgColor rgb="FFe8d5c4"/>
       </patternFill>
@@ -287,8 +293,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFc00000"/>
-        <bgColor rgb="FFc00000"/>
+        <fgColor rgb="FF2e7d32"/>
+        <bgColor rgb="FF2e7d32"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
     <fill>
@@ -299,26 +311,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFBDD7EE"/>
+        <bgColor rgb="FFBDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFed7d31"/>
         <bgColor rgb="FFed7d31"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFffeb9c"/>
-        <bgColor rgb="FFffeb9c"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF2e7d32"/>
-        <bgColor rgb="FF2e7d32"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF000000"/>
-        <bgColor rgb="FF000000"/>
+        <fgColor rgb="FFc00000"/>
+        <bgColor rgb="FFc00000"/>
       </patternFill>
     </fill>
     <fill>
@@ -496,7 +502,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -510,9 +516,6 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="30" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -522,10 +525,10 @@
     <xf numFmtId="0" fontId="19" fillId="32" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="29" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="30" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -537,16 +540,19 @@
     <xf numFmtId="0" fontId="2" fillId="32" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="33" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -556,10 +562,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="26" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="22" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="25" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -568,21 +574,24 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="34" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="34" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="35" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="35" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="35" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="36" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="22" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="25" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="36" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="37" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -633,13 +642,10 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -663,44 +669,47 @@
     <xf numFmtId="0" fontId="6" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="21" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="25" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="27" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="28" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -711,7 +720,13 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -720,28 +735,52 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="26" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="29" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="29" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="29" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="29" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="29" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="29" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="29" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1132,42 +1171,42 @@
           <t>PS5 COMPLETION PLATFORM  |  DASHBOARD - live summary (same as page 1)</t>
         </is>
       </c>
-      <c r="B1" s="89" t="n"/>
-      <c r="C1" s="89" t="n"/>
-      <c r="D1" s="89" t="n"/>
-      <c r="E1" s="89" t="n"/>
-      <c r="F1" s="89" t="n"/>
-      <c r="G1" s="89" t="n"/>
-      <c r="H1" s="89" t="n"/>
-      <c r="I1" s="89" t="n"/>
-      <c r="J1" s="90" t="n"/>
+      <c r="B1" s="100" t="n"/>
+      <c r="C1" s="100" t="n"/>
+      <c r="D1" s="100" t="n"/>
+      <c r="E1" s="100" t="n"/>
+      <c r="F1" s="100" t="n"/>
+      <c r="G1" s="100" t="n"/>
+      <c r="H1" s="100" t="n"/>
+      <c r="I1" s="100" t="n"/>
+      <c r="J1" s="101" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="8" t="n">
-        <v>23532</v>
+        <v>23537</v>
       </c>
       <c r="B2" s="9" t="n">
-        <v>9092</v>
+        <v>10354</v>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>44%</t>
         </is>
       </c>
       <c r="D2" s="11" t="n">
-        <v>2751</v>
+        <v>3094</v>
       </c>
       <c r="E2" s="9" t="n">
-        <v>521</v>
+        <v>559</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>2230</v>
+        <v>2535</v>
       </c>
       <c r="G2" s="8" t="n">
         <v>290</v>
       </c>
       <c r="H2" s="9" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
@@ -1265,15 +1304,15 @@
           <t>ITR PROGRESS BY DISCIPLINE</t>
         </is>
       </c>
-      <c r="B5" s="32" t="n"/>
-      <c r="C5" s="32" t="n"/>
-      <c r="D5" s="32" t="n"/>
-      <c r="E5" s="32" t="n"/>
-      <c r="F5" s="32" t="n"/>
-      <c r="G5" s="32" t="n"/>
-      <c r="H5" s="32" t="n"/>
-      <c r="I5" s="32" t="n"/>
-      <c r="J5" s="33" t="n"/>
+      <c r="B5" s="33" t="n"/>
+      <c r="C5" s="33" t="n"/>
+      <c r="D5" s="33" t="n"/>
+      <c r="E5" s="33" t="n"/>
+      <c r="F5" s="33" t="n"/>
+      <c r="G5" s="33" t="n"/>
+      <c r="H5" s="33" t="n"/>
+      <c r="I5" s="33" t="n"/>
+      <c r="J5" s="34" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="22" t="inlineStr">
@@ -1348,15 +1387,15 @@
         <v>2405</v>
       </c>
       <c r="D9" s="23" t="n">
-        <v>894</v>
+        <v>980</v>
       </c>
       <c r="E9" s="25" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>41%</t>
         </is>
       </c>
       <c r="F9" s="23" t="n">
-        <v>1511</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="10">
@@ -1374,15 +1413,15 @@
         <v>197</v>
       </c>
       <c r="D10" s="23" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E10" s="25" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>36%</t>
         </is>
       </c>
       <c r="F10" s="23" t="n">
-        <v>132</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11">
@@ -1397,18 +1436,18 @@
         </is>
       </c>
       <c r="C11" s="23" t="n">
-        <v>4688</v>
+        <v>4689</v>
       </c>
       <c r="D11" s="23" t="n">
-        <v>1587</v>
+        <v>1917</v>
       </c>
       <c r="E11" s="25" t="inlineStr">
         <is>
-          <t>34%</t>
+          <t>41%</t>
         </is>
       </c>
       <c r="F11" s="23" t="n">
-        <v>3101</v>
+        <v>2772</v>
       </c>
     </row>
     <row r="12">
@@ -1426,15 +1465,15 @@
         <v>263</v>
       </c>
       <c r="D12" s="23" t="n">
-        <v>94</v>
+        <v>114</v>
       </c>
       <c r="E12" s="25" t="inlineStr">
         <is>
-          <t>36%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="F12" s="23" t="n">
-        <v>169</v>
+        <v>149</v>
       </c>
     </row>
     <row r="13">
@@ -1452,15 +1491,15 @@
         <v>1530</v>
       </c>
       <c r="D13" s="23" t="n">
-        <v>964</v>
+        <v>1116</v>
       </c>
       <c r="E13" s="26" t="inlineStr">
         <is>
-          <t>63%</t>
+          <t>73%</t>
         </is>
       </c>
       <c r="F13" s="23" t="n">
-        <v>566</v>
+        <v>414</v>
       </c>
     </row>
     <row r="14">
@@ -1504,7 +1543,7 @@
         <v>3021</v>
       </c>
       <c r="D15" s="23" t="n">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="E15" s="25" t="inlineStr">
         <is>
@@ -1512,7 +1551,7 @@
         </is>
       </c>
       <c r="F15" s="23" t="n">
-        <v>2538</v>
+        <v>2537</v>
       </c>
     </row>
     <row r="16">
@@ -1527,18 +1566,18 @@
         </is>
       </c>
       <c r="C16" s="27" t="n">
-        <v>12284</v>
+        <v>12285</v>
       </c>
       <c r="D16" s="27" t="n">
-        <v>4095</v>
+        <v>4689</v>
       </c>
       <c r="E16" s="25" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>8189</v>
+        <v>7596</v>
       </c>
     </row>
     <row r="17">
@@ -1579,18 +1618,18 @@
         </is>
       </c>
       <c r="C18" s="23" t="n">
-        <v>5888</v>
+        <v>5889</v>
       </c>
       <c r="D18" s="23" t="n">
-        <v>1947</v>
+        <v>2186</v>
       </c>
       <c r="E18" s="25" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>37%</t>
         </is>
       </c>
       <c r="F18" s="23" t="n">
-        <v>3941</v>
+        <v>3703</v>
       </c>
     </row>
     <row r="19">
@@ -1631,18 +1670,18 @@
         </is>
       </c>
       <c r="C20" s="23" t="n">
-        <v>2454</v>
+        <v>2456</v>
       </c>
       <c r="D20" s="23" t="n">
-        <v>1133</v>
-      </c>
-      <c r="E20" s="25" t="inlineStr">
-        <is>
-          <t>46%</t>
+        <v>1409</v>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>57%</t>
         </is>
       </c>
       <c r="F20" s="23" t="n">
-        <v>1321</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="21">
@@ -1660,15 +1699,15 @@
         <v>553</v>
       </c>
       <c r="D21" s="23" t="n">
-        <v>290</v>
+        <v>304</v>
       </c>
       <c r="E21" s="26" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>55%</t>
         </is>
       </c>
       <c r="F21" s="23" t="n">
-        <v>263</v>
+        <v>249</v>
       </c>
     </row>
     <row r="22">
@@ -1686,15 +1725,15 @@
         <v>1656</v>
       </c>
       <c r="D22" s="23" t="n">
-        <v>1263</v>
+        <v>1351</v>
       </c>
       <c r="E22" s="26" t="inlineStr">
         <is>
-          <t>76%</t>
+          <t>82%</t>
         </is>
       </c>
       <c r="F22" s="23" t="n">
-        <v>393</v>
+        <v>305</v>
       </c>
     </row>
     <row r="23">
@@ -1738,7 +1777,7 @@
         <v>272</v>
       </c>
       <c r="D24" s="23" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E24" s="26" t="inlineStr">
         <is>
@@ -1746,7 +1785,7 @@
         </is>
       </c>
       <c r="F24" s="23" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="25">
@@ -1761,18 +1800,18 @@
         </is>
       </c>
       <c r="C25" s="27" t="n">
-        <v>10823</v>
+        <v>10826</v>
       </c>
       <c r="D25" s="27" t="n">
-        <v>4784</v>
-      </c>
-      <c r="E25" s="25" t="inlineStr">
-        <is>
-          <t>44%</t>
+        <v>5402</v>
+      </c>
+      <c r="E25" s="26" t="inlineStr">
+        <is>
+          <t>50%</t>
         </is>
       </c>
       <c r="F25" s="27" t="n">
-        <v>6039</v>
+        <v>5424</v>
       </c>
     </row>
     <row r="26">
@@ -1790,15 +1829,15 @@
         <v>74</v>
       </c>
       <c r="D26" s="23" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E26" s="25" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="F26" s="23" t="n">
-        <v>71</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27">
@@ -1868,15 +1907,15 @@
         <v>200</v>
       </c>
       <c r="D29" s="23" t="n">
-        <v>151</v>
-      </c>
-      <c r="E29" s="26" t="inlineStr">
-        <is>
-          <t>76%</t>
+        <v>192</v>
+      </c>
+      <c r="E29" s="29" t="inlineStr">
+        <is>
+          <t>96%</t>
         </is>
       </c>
       <c r="F29" s="23" t="n">
-        <v>49</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30">
@@ -1920,15 +1959,15 @@
         <v>66</v>
       </c>
       <c r="D31" s="23" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E31" s="26" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>53%</t>
         </is>
       </c>
       <c r="F31" s="23" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="32">
@@ -1998,41 +2037,41 @@
         <v>397</v>
       </c>
       <c r="D34" s="27" t="n">
-        <v>193</v>
-      </c>
-      <c r="E34" s="25" t="inlineStr">
-        <is>
-          <t>49%</t>
+        <v>243</v>
+      </c>
+      <c r="E34" s="26" t="inlineStr">
+        <is>
+          <t>61%</t>
         </is>
       </c>
       <c r="F34" s="27" t="n">
-        <v>204</v>
+        <v>154</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="29" t="inlineStr">
+      <c r="A35" s="30" t="inlineStr">
         <is>
           <t>Grand</t>
         </is>
       </c>
-      <c r="B35" s="30" t="inlineStr">
+      <c r="B35" s="31" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C35" s="29" t="n">
-        <v>23532</v>
-      </c>
-      <c r="D35" s="29" t="n">
-        <v>9092</v>
-      </c>
-      <c r="E35" s="25" t="inlineStr">
-        <is>
-          <t>39%</t>
-        </is>
-      </c>
-      <c r="F35" s="29" t="n">
-        <v>14440</v>
+      <c r="C35" s="30" t="n">
+        <v>15480</v>
+      </c>
+      <c r="D35" s="30" t="n">
+        <v>8254</v>
+      </c>
+      <c r="E35" s="26" t="inlineStr">
+        <is>
+          <t>53%</t>
+        </is>
+      </c>
+      <c r="F35" s="30" t="n">
+        <v>7226</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
@@ -2041,15 +2080,15 @@
           <t>PUNCH SUMMARY (A / B / C)</t>
         </is>
       </c>
-      <c r="B38" s="32" t="n"/>
-      <c r="C38" s="32" t="n"/>
-      <c r="D38" s="32" t="n"/>
-      <c r="E38" s="32" t="n"/>
-      <c r="F38" s="32" t="n"/>
-      <c r="G38" s="32" t="n"/>
-      <c r="H38" s="32" t="n"/>
-      <c r="I38" s="32" t="n"/>
-      <c r="J38" s="33" t="n"/>
+      <c r="B38" s="33" t="n"/>
+      <c r="C38" s="33" t="n"/>
+      <c r="D38" s="33" t="n"/>
+      <c r="E38" s="33" t="n"/>
+      <c r="F38" s="33" t="n"/>
+      <c r="G38" s="33" t="n"/>
+      <c r="H38" s="33" t="n"/>
+      <c r="I38" s="33" t="n"/>
+      <c r="J38" s="34" t="n"/>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="22" t="inlineStr">
@@ -2057,27 +2096,27 @@
           <t>DISCIPLINE</t>
         </is>
       </c>
-      <c r="B39" s="31" t="inlineStr">
+      <c r="B39" s="32" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C39" s="32" t="n"/>
-      <c r="D39" s="33" t="n"/>
-      <c r="E39" s="34" t="inlineStr">
+      <c r="C39" s="33" t="n"/>
+      <c r="D39" s="34" t="n"/>
+      <c r="E39" s="35" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="F39" s="32" t="n"/>
-      <c r="G39" s="33" t="n"/>
-      <c r="H39" s="35" t="inlineStr">
+      <c r="F39" s="33" t="n"/>
+      <c r="G39" s="34" t="n"/>
+      <c r="H39" s="36" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="I39" s="32" t="n"/>
-      <c r="J39" s="33" t="n"/>
+      <c r="I39" s="33" t="n"/>
+      <c r="J39" s="34" t="n"/>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="22" t="inlineStr"/>
@@ -2168,31 +2207,31 @@
         </is>
       </c>
       <c r="B42" s="23" t="n">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C42" s="23" t="n">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D42" s="23" t="n">
         <v>161</v>
       </c>
       <c r="E42" s="23" t="n">
-        <v>358</v>
+        <v>400</v>
       </c>
       <c r="F42" s="23" t="n">
         <v>11</v>
       </c>
       <c r="G42" s="23" t="n">
-        <v>347</v>
+        <v>389</v>
       </c>
       <c r="H42" s="23" t="n">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="I42" s="23" t="n">
         <v>16</v>
       </c>
       <c r="J42" s="23" t="n">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="43">
@@ -2211,13 +2250,13 @@
         <v>2</v>
       </c>
       <c r="E43" s="23" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F43" s="23" t="n">
         <v>0</v>
       </c>
       <c r="G43" s="23" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H43" s="23" t="n">
         <v>0</v>
@@ -2245,22 +2284,22 @@
         <v>8</v>
       </c>
       <c r="E44" s="23" t="n">
-        <v>215</v>
+        <v>312</v>
       </c>
       <c r="F44" s="23" t="n">
         <v>20</v>
       </c>
       <c r="G44" s="23" t="n">
-        <v>195</v>
+        <v>292</v>
       </c>
       <c r="H44" s="23" t="n">
-        <v>43</v>
+        <v>92</v>
       </c>
       <c r="I44" s="23" t="n">
         <v>5</v>
       </c>
       <c r="J44" s="23" t="n">
-        <v>38</v>
+        <v>87</v>
       </c>
     </row>
     <row r="45">
@@ -2270,31 +2309,31 @@
         </is>
       </c>
       <c r="B45" s="23" t="n">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C45" s="23" t="n">
         <v>133</v>
       </c>
       <c r="D45" s="23" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E45" s="23" t="n">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="F45" s="23" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G45" s="23" t="n">
-        <v>240</v>
+        <v>251</v>
       </c>
       <c r="H45" s="23" t="n">
-        <v>338</v>
+        <v>357</v>
       </c>
       <c r="I45" s="23" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J45" s="23" t="n">
-        <v>259</v>
+        <v>277</v>
       </c>
     </row>
     <row r="46">
@@ -2307,28 +2346,28 @@
         <v>12</v>
       </c>
       <c r="C46" s="23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D46" s="23" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E46" s="23" t="n">
-        <v>669</v>
+        <v>733</v>
       </c>
       <c r="F46" s="23" t="n">
-        <v>262</v>
+        <v>340</v>
       </c>
       <c r="G46" s="23" t="n">
-        <v>407</v>
+        <v>393</v>
       </c>
       <c r="H46" s="23" t="n">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="I46" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J46" s="23" t="n">
-        <v>6</v>
+        <v>42</v>
       </c>
     </row>
     <row r="47">
@@ -2400,37 +2439,37 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="30" t="inlineStr">
+      <c r="A49" s="31" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B49" s="29" t="n">
-        <v>669</v>
-      </c>
-      <c r="C49" s="29" t="n">
-        <v>430</v>
-      </c>
-      <c r="D49" s="29" t="n">
-        <v>239</v>
-      </c>
-      <c r="E49" s="29" t="n">
-        <v>1554</v>
-      </c>
-      <c r="F49" s="29" t="n">
-        <v>344</v>
-      </c>
-      <c r="G49" s="29" t="n">
-        <v>1210</v>
-      </c>
-      <c r="H49" s="29" t="n">
-        <v>524</v>
-      </c>
-      <c r="I49" s="29" t="n">
-        <v>106</v>
-      </c>
-      <c r="J49" s="29" t="n">
-        <v>418</v>
+      <c r="B49" s="30" t="n">
+        <v>672</v>
+      </c>
+      <c r="C49" s="30" t="n">
+        <v>429</v>
+      </c>
+      <c r="D49" s="30" t="n">
+        <v>243</v>
+      </c>
+      <c r="E49" s="30" t="n">
+        <v>1771</v>
+      </c>
+      <c r="F49" s="30" t="n">
+        <v>423</v>
+      </c>
+      <c r="G49" s="30" t="n">
+        <v>1348</v>
+      </c>
+      <c r="H49" s="30" t="n">
+        <v>648</v>
+      </c>
+      <c r="I49" s="30" t="n">
+        <v>108</v>
+      </c>
+      <c r="J49" s="30" t="n">
+        <v>540</v>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1">
@@ -2439,15 +2478,15 @@
           <t>MILESTONE &amp; DIS - 290 ROWS</t>
         </is>
       </c>
-      <c r="B52" s="32" t="n"/>
-      <c r="C52" s="32" t="n"/>
-      <c r="D52" s="32" t="n"/>
-      <c r="E52" s="32" t="n"/>
-      <c r="F52" s="32" t="n"/>
-      <c r="G52" s="32" t="n"/>
-      <c r="H52" s="32" t="n"/>
-      <c r="I52" s="32" t="n"/>
-      <c r="J52" s="33" t="n"/>
+      <c r="B52" s="33" t="n"/>
+      <c r="C52" s="33" t="n"/>
+      <c r="D52" s="33" t="n"/>
+      <c r="E52" s="33" t="n"/>
+      <c r="F52" s="33" t="n"/>
+      <c r="G52" s="33" t="n"/>
+      <c r="H52" s="33" t="n"/>
+      <c r="I52" s="33" t="n"/>
+      <c r="J52" s="34" t="n"/>
     </row>
     <row r="53" ht="22" customHeight="1">
       <c r="A53" s="22" t="inlineStr">
@@ -2507,7 +2546,7 @@
           <t>PS5-01-01</t>
         </is>
       </c>
-      <c r="B54" s="36" t="inlineStr">
+      <c r="B54" s="37" t="inlineStr">
         <is>
           <t>PS5-01-01 - Fire Water Jockey Pump A/B</t>
         </is>
@@ -2535,7 +2574,7 @@
           <t>PS5-01-02</t>
         </is>
       </c>
-      <c r="B55" s="36" t="inlineStr">
+      <c r="B55" s="37" t="inlineStr">
         <is>
           <t>PS5-01-02 - Fire Water Pump A</t>
         </is>
@@ -2563,7 +2602,7 @@
           <t>PS5-01-03</t>
         </is>
       </c>
-      <c r="B56" s="36" t="inlineStr">
+      <c r="B56" s="37" t="inlineStr">
         <is>
           <t>PS5-01-03 - Fire Water Pump B</t>
         </is>
@@ -2591,7 +2630,7 @@
           <t>PS5-01-04</t>
         </is>
       </c>
-      <c r="B57" s="36" t="inlineStr">
+      <c r="B57" s="37" t="inlineStr">
         <is>
           <t>PS5-01-04 - Fire Water Pump Mini Flow Recycle</t>
         </is>
@@ -2619,7 +2658,7 @@
           <t>PS5-01-05</t>
         </is>
       </c>
-      <c r="B58" s="36" t="inlineStr">
+      <c r="B58" s="37" t="inlineStr">
         <is>
           <t>PS5-01-05 - Foam Skid</t>
         </is>
@@ -2647,7 +2686,7 @@
           <t>PS5-01-06</t>
         </is>
       </c>
-      <c r="B59" s="36" t="inlineStr">
+      <c r="B59" s="37" t="inlineStr">
         <is>
           <t>PS5-01-06 - Foam Concentrate Distribution</t>
         </is>
@@ -2675,7 +2714,7 @@
           <t>PS5-01-07</t>
         </is>
       </c>
-      <c r="B60" s="36" t="inlineStr">
+      <c r="B60" s="37" t="inlineStr">
         <is>
           <t>PS5-01-07 - Fire Water Ring Main &amp; Distribution</t>
         </is>
@@ -2703,7 +2742,7 @@
           <t>PS5-01-08</t>
         </is>
       </c>
-      <c r="B61" s="36" t="inlineStr">
+      <c r="B61" s="37" t="inlineStr">
         <is>
           <t>PS5-01-08 - PS5 Deluge Valve Skid (PS5-01-UK-6100)</t>
         </is>
@@ -2731,7 +2770,7 @@
           <t>PS5-01-09</t>
         </is>
       </c>
-      <c r="B62" s="36" t="inlineStr">
+      <c r="B62" s="37" t="inlineStr">
         <is>
           <t>PS5-01-09 - Inergen for EITS Building</t>
         </is>
@@ -2759,7 +2798,7 @@
           <t>PS5-01-10</t>
         </is>
       </c>
-      <c r="B63" s="36" t="inlineStr">
+      <c r="B63" s="37" t="inlineStr">
         <is>
           <t>PS5-01-10 - Water Mist Package</t>
         </is>
@@ -2787,7 +2826,7 @@
           <t>PS5-01-11</t>
         </is>
       </c>
-      <c r="B64" s="36" t="inlineStr">
+      <c r="B64" s="37" t="inlineStr">
         <is>
           <t>PS5-01-11 - Inergen for Power Gen Building</t>
         </is>
@@ -2815,7 +2854,7 @@
           <t>PS5-02-01</t>
         </is>
       </c>
-      <c r="B65" s="36" t="inlineStr">
+      <c r="B65" s="37" t="inlineStr">
         <is>
           <t>PS5-02-01 - Miscellaneous Safety equipment</t>
         </is>
@@ -2843,7 +2882,7 @@
           <t>PS5-02-02</t>
         </is>
       </c>
-      <c r="B66" s="36" t="inlineStr">
+      <c r="B66" s="37" t="inlineStr">
         <is>
           <t>PS5-02-02 - Portable Fire Fighting Equipments</t>
         </is>
@@ -2871,7 +2910,7 @@
           <t>PS5-03-01</t>
         </is>
       </c>
-      <c r="B67" s="36" t="inlineStr">
+      <c r="B67" s="37" t="inlineStr">
         <is>
           <t>PS5-03-01 - FZ-01 - Process Area</t>
         </is>
@@ -2899,7 +2938,7 @@
           <t>PS5-03-03</t>
         </is>
       </c>
-      <c r="B68" s="36" t="inlineStr">
+      <c r="B68" s="37" t="inlineStr">
         <is>
           <t>PS5-03-03 - FZ-03 - Buildings Area</t>
         </is>
@@ -2927,7 +2966,7 @@
           <t>PS5-03-04</t>
         </is>
       </c>
-      <c r="B69" s="36" t="inlineStr">
+      <c r="B69" s="37" t="inlineStr">
         <is>
           <t>PS5-03-04 - FZ-04 - Utilities - Diesel and Firewater Pumps Areas</t>
         </is>
@@ -2955,7 +2994,7 @@
           <t>PS5-03-06</t>
         </is>
       </c>
-      <c r="B70" s="36" t="inlineStr">
+      <c r="B70" s="37" t="inlineStr">
         <is>
           <t>PS5-03-06 - FZ-06 - Transformer Area</t>
         </is>
@@ -2983,7 +3022,7 @@
           <t>PS5-03-07</t>
         </is>
       </c>
-      <c r="B71" s="36" t="inlineStr">
+      <c r="B71" s="37" t="inlineStr">
         <is>
           <t>PS5-03-07 - FZ-07 - Pretreatment Area</t>
         </is>
@@ -3011,7 +3050,7 @@
           <t>PS5-03-08</t>
         </is>
       </c>
-      <c r="B72" s="36" t="inlineStr">
+      <c r="B72" s="37" t="inlineStr">
         <is>
           <t>PS5-03-08 - FZ-08 - Utilities - Power Generation Area - External</t>
         </is>
@@ -3039,7 +3078,7 @@
           <t>PS5-03-09</t>
         </is>
       </c>
-      <c r="B73" s="36" t="inlineStr">
+      <c r="B73" s="37" t="inlineStr">
         <is>
           <t>PS5-03-09 - FZ-09 - Power Generation Building - Engine Bay 1</t>
         </is>
@@ -3067,7 +3106,7 @@
           <t>PS5-03-10</t>
         </is>
       </c>
-      <c r="B74" s="36" t="inlineStr">
+      <c r="B74" s="37" t="inlineStr">
         <is>
           <t>PS5-03-10 - FZ-10 - Power Generation Building - Engine Bay 2</t>
         </is>
@@ -3095,7 +3134,7 @@
           <t>PS5-03-11</t>
         </is>
       </c>
-      <c r="B75" s="36" t="inlineStr">
+      <c r="B75" s="37" t="inlineStr">
         <is>
           <t>PS5-03-11 - FZ-11 - Power Generation Building - Engine Bay 3</t>
         </is>
@@ -3123,7 +3162,7 @@
           <t>PS5-03-12</t>
         </is>
       </c>
-      <c r="B76" s="36" t="inlineStr">
+      <c r="B76" s="37" t="inlineStr">
         <is>
           <t>PS5-03-12 - FZ-12 - Power Generation Building - Engine Bay 4</t>
         </is>
@@ -3151,7 +3190,7 @@
           <t>PS5-03-13</t>
         </is>
       </c>
-      <c r="B77" s="36" t="inlineStr">
+      <c r="B77" s="37" t="inlineStr">
         <is>
           <t>PS5-03-13 - FZ-13 - Power Generation Building - Instrument Air Room</t>
         </is>
@@ -3179,7 +3218,7 @@
           <t>PS5-03-14</t>
         </is>
       </c>
-      <c r="B78" s="36" t="inlineStr">
+      <c r="B78" s="37" t="inlineStr">
         <is>
           <t>PS5-03-14 - FZ-14 - Power Generation Building - Switchgear Room</t>
         </is>
@@ -3207,7 +3246,7 @@
           <t>PS5-03-15</t>
         </is>
       </c>
-      <c r="B79" s="36" t="inlineStr">
+      <c r="B79" s="37" t="inlineStr">
         <is>
           <t>PS5-03-15 - FZ-15 - Power Generation Building - Generator Room 1</t>
         </is>
@@ -3235,7 +3274,7 @@
           <t>PS5-03-16</t>
         </is>
       </c>
-      <c r="B80" s="36" t="inlineStr">
+      <c r="B80" s="37" t="inlineStr">
         <is>
           <t>PS5-03-16 - FZ-16 - Power Generation Building - Generator Room 2</t>
         </is>
@@ -3263,7 +3302,7 @@
           <t>PS5-03-17</t>
         </is>
       </c>
-      <c r="B81" s="36" t="inlineStr">
+      <c r="B81" s="37" t="inlineStr">
         <is>
           <t>PS5-03-17 - FZ-17 - Power Generation Building - Generator Room 3</t>
         </is>
@@ -3291,7 +3330,7 @@
           <t>PS5-03-18</t>
         </is>
       </c>
-      <c r="B82" s="36" t="inlineStr">
+      <c r="B82" s="37" t="inlineStr">
         <is>
           <t>PS5-03-18 - FZ-18 - Power Generation Building - Generator Room 4</t>
         </is>
@@ -3319,7 +3358,7 @@
           <t>PS5-03-19</t>
         </is>
       </c>
-      <c r="B83" s="36" t="inlineStr">
+      <c r="B83" s="37" t="inlineStr">
         <is>
           <t>PS5-03-19 - FZ-19 - Power Generation Building - Battery Room</t>
         </is>
@@ -3347,7 +3386,7 @@
           <t>PS5-03-20</t>
         </is>
       </c>
-      <c r="B84" s="36" t="inlineStr">
+      <c r="B84" s="37" t="inlineStr">
         <is>
           <t>PS5-03-20 - FZ-20 - Emergency Diesel Generator Enclosure</t>
         </is>
@@ -3375,7 +3414,7 @@
           <t>PS5-03-21</t>
         </is>
       </c>
-      <c r="B85" s="36" t="inlineStr">
+      <c r="B85" s="37" t="inlineStr">
         <is>
           <t>PS5-03-21 - FZ-21 - Power Generation Building - Air Handling Unit</t>
         </is>
@@ -3403,7 +3442,7 @@
           <t>PS5-03-22</t>
         </is>
       </c>
-      <c r="B86" s="36" t="inlineStr">
+      <c r="B86" s="37" t="inlineStr">
         <is>
           <t>PS5-03-22 - FZ-G1 - Guard House</t>
         </is>
@@ -3431,7 +3470,7 @@
           <t>PS5-03-23</t>
         </is>
       </c>
-      <c r="B87" s="36" t="inlineStr">
+      <c r="B87" s="37" t="inlineStr">
         <is>
           <t>PS5-03-23 - FZ-E1 to E3 - EITS Building</t>
         </is>
@@ -3459,7 +3498,7 @@
           <t>PS5-03-24</t>
         </is>
       </c>
-      <c r="B88" s="36" t="inlineStr">
+      <c r="B88" s="37" t="inlineStr">
         <is>
           <t>PS5-03-24 - FZ - Office and Facilities Building</t>
         </is>
@@ -3487,7 +3526,7 @@
           <t>PS5-03-25</t>
         </is>
       </c>
-      <c r="B89" s="36" t="inlineStr">
+      <c r="B89" s="37" t="inlineStr">
         <is>
           <t>PS5-03-25 - FZ - Workshop &amp; Warehouse</t>
         </is>
@@ -3515,7 +3554,7 @@
           <t>PS5-04-01</t>
         </is>
       </c>
-      <c r="B90" s="36" t="inlineStr">
+      <c r="B90" s="37" t="inlineStr">
         <is>
           <t>PS5-04-01 - Office Building PCS System</t>
         </is>
@@ -3543,7 +3582,7 @@
           <t>PS5-04-02</t>
         </is>
       </c>
-      <c r="B91" s="36" t="inlineStr">
+      <c r="B91" s="37" t="inlineStr">
         <is>
           <t>PS5-04-02 - Office Building SIS/FGS System</t>
         </is>
@@ -3571,7 +3610,7 @@
           <t>PS5-04-03</t>
         </is>
       </c>
-      <c r="B92" s="36" t="inlineStr">
+      <c r="B92" s="37" t="inlineStr">
         <is>
           <t>PS5-04-03 - 33kV ICSS System</t>
         </is>
@@ -3599,7 +3638,7 @@
           <t>PS5-04-04</t>
         </is>
       </c>
-      <c r="B93" s="36" t="inlineStr">
+      <c r="B93" s="37" t="inlineStr">
         <is>
           <t>PS5-04-04 - 33kV PCS System</t>
         </is>
@@ -3627,7 +3666,7 @@
           <t>PS5-04-05</t>
         </is>
       </c>
-      <c r="B94" s="36" t="inlineStr">
+      <c r="B94" s="37" t="inlineStr">
         <is>
           <t>PS5-04-05 - 33kV SIS/FGS System</t>
         </is>
@@ -3655,7 +3694,7 @@
           <t>PS5-05-01</t>
         </is>
       </c>
-      <c r="B95" s="36" t="inlineStr">
+      <c r="B95" s="37" t="inlineStr">
         <is>
           <t>PS5-05-01 - Emergency Diesel Generator Package</t>
         </is>
@@ -3683,7 +3722,7 @@
           <t>PS5-05-02</t>
         </is>
       </c>
-      <c r="B96" s="36" t="inlineStr">
+      <c r="B96" s="37" t="inlineStr">
         <is>
           <t>PS5-05-02 - Emergency Diesel Generator Package (UCP)</t>
         </is>
@@ -3711,7 +3750,7 @@
           <t>PS5-06-01</t>
         </is>
       </c>
-      <c r="B97" s="36" t="inlineStr">
+      <c r="B97" s="37" t="inlineStr">
         <is>
           <t>PS5-06-01 - AC UPS - EITS Building</t>
         </is>
@@ -3739,7 +3778,7 @@
           <t>PS5-06-02</t>
         </is>
       </c>
-      <c r="B98" s="36" t="inlineStr">
+      <c r="B98" s="37" t="inlineStr">
         <is>
           <t>PS5-06-02 - AC UPS - Power Generator Building</t>
         </is>
@@ -3767,7 +3806,7 @@
           <t>PS5-06-03</t>
         </is>
       </c>
-      <c r="B99" s="36" t="inlineStr">
+      <c r="B99" s="37" t="inlineStr">
         <is>
           <t>PS5-06-03 - AC UPS - Office &amp; Facilities Building</t>
         </is>
@@ -3795,7 +3834,7 @@
           <t>PS5-06-04</t>
         </is>
       </c>
-      <c r="B100" s="36" t="inlineStr">
+      <c r="B100" s="37" t="inlineStr">
         <is>
           <t>PS5-06-04 - AC UPS - Guard House</t>
         </is>
@@ -3823,7 +3862,7 @@
           <t>PS5-06-05</t>
         </is>
       </c>
-      <c r="B101" s="36" t="inlineStr">
+      <c r="B101" s="37" t="inlineStr">
         <is>
           <t>PS5-06-05 - AC UPS - Workshop &amp; Warehouse</t>
         </is>
@@ -3851,7 +3890,7 @@
           <t>PS5-08-01</t>
         </is>
       </c>
-      <c r="B102" s="36" t="inlineStr">
+      <c r="B102" s="37" t="inlineStr">
         <is>
           <t>PS5-08-01 - PAGA</t>
         </is>
@@ -3879,7 +3918,7 @@
           <t>PS5-08-03</t>
         </is>
       </c>
-      <c r="B103" s="36" t="inlineStr">
+      <c r="B103" s="37" t="inlineStr">
         <is>
           <t>PS5-08-03 - Telephone</t>
         </is>
@@ -3907,7 +3946,7 @@
           <t>PS5-08-04</t>
         </is>
       </c>
-      <c r="B104" s="36" t="inlineStr">
+      <c r="B104" s="37" t="inlineStr">
         <is>
           <t>PS5-08-04 - Hotline</t>
         </is>
@@ -3935,7 +3974,7 @@
           <t>PS5-08-07</t>
         </is>
       </c>
-      <c r="B105" s="36" t="inlineStr">
+      <c r="B105" s="37" t="inlineStr">
         <is>
           <t>PS5-08-07 - Multi-Channel Voice Recorder</t>
         </is>
@@ -3963,7 +4002,7 @@
           <t>PS5-08-11</t>
         </is>
       </c>
-      <c r="B106" s="36" t="inlineStr">
+      <c r="B106" s="37" t="inlineStr">
         <is>
           <t>PS5-08-11 - Corporate LAN  (SIE)</t>
         </is>
@@ -3991,7 +4030,7 @@
           <t>PS5-08-12</t>
         </is>
       </c>
-      <c r="B107" s="36" t="inlineStr">
+      <c r="B107" s="37" t="inlineStr">
         <is>
           <t>PS5-08-12 - Corporate Wireless LAN (SIE)</t>
         </is>
@@ -4019,7 +4058,7 @@
           <t>PS5-08-13</t>
         </is>
       </c>
-      <c r="B108" s="36" t="inlineStr">
+      <c r="B108" s="37" t="inlineStr">
         <is>
           <t>PS5-08-13 - Safety Data Network (SII SP3 SAF)</t>
         </is>
@@ -4047,7 +4086,7 @@
           <t>PS5-08-14</t>
         </is>
       </c>
-      <c r="B109" s="36" t="inlineStr">
+      <c r="B109" s="37" t="inlineStr">
         <is>
           <t>PS5-08-14 - Industrial Data Network (SII SP1)</t>
         </is>
@@ -4075,7 +4114,7 @@
           <t>PS5-08-15</t>
         </is>
       </c>
-      <c r="B110" s="36" t="inlineStr">
+      <c r="B110" s="37" t="inlineStr">
         <is>
           <t>PS5-08-15 - Security Data Network (SII SP3 SEC)</t>
         </is>
@@ -4103,7 +4142,7 @@
           <t>PS5-08-23</t>
         </is>
       </c>
-      <c r="B111" s="36" t="inlineStr">
+      <c r="B111" s="37" t="inlineStr">
         <is>
           <t>PS5-08-23 - VHF Trunk Radio System</t>
         </is>
@@ -4131,7 +4170,7 @@
           <t>PS5-08-34</t>
         </is>
       </c>
-      <c r="B112" s="36" t="inlineStr">
+      <c r="B112" s="37" t="inlineStr">
         <is>
           <t>PS5-08-34 - Satphone</t>
         </is>
@@ -4159,7 +4198,7 @@
           <t>PS5-08-35</t>
         </is>
       </c>
-      <c r="B113" s="36" t="inlineStr">
+      <c r="B113" s="37" t="inlineStr">
         <is>
           <t>PS5-08-35 - Optical Transport Network</t>
         </is>
@@ -4187,7 +4226,7 @@
           <t>PS5-08-36</t>
         </is>
       </c>
-      <c r="B114" s="36" t="inlineStr">
+      <c r="B114" s="37" t="inlineStr">
         <is>
           <t>PS5-08-36 - Pipeline FO Cable &amp; EPRS</t>
         </is>
@@ -4215,7 +4254,7 @@
           <t>PS5-08-51</t>
         </is>
       </c>
-      <c r="B115" s="36" t="inlineStr">
+      <c r="B115" s="37" t="inlineStr">
         <is>
           <t>PS5-08-51 - Entertainment</t>
         </is>
@@ -4243,7 +4282,7 @@
           <t>PS5-08-52</t>
         </is>
       </c>
-      <c r="B116" s="36" t="inlineStr">
+      <c r="B116" s="37" t="inlineStr">
         <is>
           <t>PS5-08-52 - Process &amp; Security CCTV</t>
         </is>
@@ -4271,7 +4310,7 @@
           <t>PS5-08-55</t>
         </is>
       </c>
-      <c r="B117" s="36" t="inlineStr">
+      <c r="B117" s="37" t="inlineStr">
         <is>
           <t>PS5-08-55 - Videoconference</t>
         </is>
@@ -4299,7 +4338,7 @@
           <t>PS5-08-61</t>
         </is>
       </c>
-      <c r="B118" s="36" t="inlineStr">
+      <c r="B118" s="37" t="inlineStr">
         <is>
           <t>PS5-08-61 - Meteocean</t>
         </is>
@@ -4327,7 +4366,7 @@
           <t>PS5-08-71</t>
         </is>
       </c>
-      <c r="B119" s="36" t="inlineStr">
+      <c r="B119" s="37" t="inlineStr">
         <is>
           <t>PS5-08-71 - Structured Cabling (CAT6)</t>
         </is>
@@ -4355,7 +4394,7 @@
           <t>PS5-08-72</t>
         </is>
       </c>
-      <c r="B120" s="36" t="inlineStr">
+      <c r="B120" s="37" t="inlineStr">
         <is>
           <t>PS5-08-72 - Structured Cabling (FO)</t>
         </is>
@@ -4383,7 +4422,7 @@
           <t>PS5-08-81</t>
         </is>
       </c>
-      <c r="B121" s="36" t="inlineStr">
+      <c r="B121" s="37" t="inlineStr">
         <is>
           <t>PS5-08-81 - Guard tour</t>
         </is>
@@ -4411,7 +4450,7 @@
           <t>PS5-08-82</t>
         </is>
       </c>
-      <c r="B122" s="36" t="inlineStr">
+      <c r="B122" s="37" t="inlineStr">
         <is>
           <t>PS5-08-82 - Key Management</t>
         </is>
@@ -4439,7 +4478,7 @@
           <t>PS5-08-83</t>
         </is>
       </c>
-      <c r="B123" s="36" t="inlineStr">
+      <c r="B123" s="37" t="inlineStr">
         <is>
           <t>PS5-08-83 - Perimeter &amp; Pipeline intrusion detection system</t>
         </is>
@@ -4467,7 +4506,7 @@
           <t>PS5-08-85</t>
         </is>
       </c>
-      <c r="B124" s="36" t="inlineStr">
+      <c r="B124" s="37" t="inlineStr">
         <is>
           <t>PS5-08-85 - Access Control, POB &amp; e-Mustering</t>
         </is>
@@ -4495,7 +4534,7 @@
           <t>PS5-08-86</t>
         </is>
       </c>
-      <c r="B125" s="36" t="inlineStr">
+      <c r="B125" s="37" t="inlineStr">
         <is>
           <t>PS5-08-86 - Integrated Security Management System</t>
         </is>
@@ -4523,7 +4562,7 @@
           <t>PS5-08-92</t>
         </is>
       </c>
-      <c r="B126" s="36" t="inlineStr">
+      <c r="B126" s="37" t="inlineStr">
         <is>
           <t>PS5-08-92 - Telecom Mast</t>
         </is>
@@ -4551,7 +4590,7 @@
           <t>PS5-08-93</t>
         </is>
       </c>
-      <c r="B127" s="36" t="inlineStr">
+      <c r="B127" s="37" t="inlineStr">
         <is>
           <t>PS5-08-93 - Telecom Monitoring System</t>
         </is>
@@ -4579,7 +4618,7 @@
           <t>PS5-09-01</t>
         </is>
       </c>
-      <c r="B128" s="36" t="inlineStr">
+      <c r="B128" s="37" t="inlineStr">
         <is>
           <t>PS5-09-01 - HVAC for Office and Facilities building</t>
         </is>
@@ -4607,7 +4646,7 @@
           <t>PS5-09-02</t>
         </is>
       </c>
-      <c r="B129" s="36" t="inlineStr">
+      <c r="B129" s="37" t="inlineStr">
         <is>
           <t>PS5-09-02 - HVAC for Guard House</t>
         </is>
@@ -4635,7 +4674,7 @@
           <t>PS5-09-03</t>
         </is>
       </c>
-      <c r="B130" s="36" t="inlineStr">
+      <c r="B130" s="37" t="inlineStr">
         <is>
           <t>PS5-09-03 - HVAC for Generator Building</t>
         </is>
@@ -4663,7 +4702,7 @@
           <t>PS5-09-04</t>
         </is>
       </c>
-      <c r="B131" s="36" t="inlineStr">
+      <c r="B131" s="37" t="inlineStr">
         <is>
           <t>PS5-09-04 - HVAC for Workshop &amp; Warehouse</t>
         </is>
@@ -4691,7 +4730,7 @@
           <t>PS5-09-05</t>
         </is>
       </c>
-      <c r="B132" s="36" t="inlineStr">
+      <c r="B132" s="37" t="inlineStr">
         <is>
           <t>PS5-09-05 - HVAC for EITS Building</t>
         </is>
@@ -4719,7 +4758,7 @@
           <t>PS5-0H-01</t>
         </is>
       </c>
-      <c r="B133" s="36" t="inlineStr">
+      <c r="B133" s="37" t="inlineStr">
         <is>
           <t>PS5-0H-01 - HIPPS</t>
         </is>
@@ -4747,7 +4786,7 @@
           <t>PS5-25-01</t>
         </is>
       </c>
-      <c r="B134" s="36" t="inlineStr">
+      <c r="B134" s="37" t="inlineStr">
         <is>
           <t>PS5-25-01 - Export Pipeline Pig Receiver</t>
         </is>
@@ -4775,7 +4814,7 @@
           <t>PS5-25-02</t>
         </is>
       </c>
-      <c r="B135" s="36" t="inlineStr">
+      <c r="B135" s="37" t="inlineStr">
         <is>
           <t>PS5-25-02 - Crude Oil Export Pump A</t>
         </is>
@@ -4803,7 +4842,7 @@
           <t>PS5-25-03</t>
         </is>
       </c>
-      <c r="B136" s="36" t="inlineStr">
+      <c r="B136" s="37" t="inlineStr">
         <is>
           <t>PS5-25-03 - Crude Oil Export Pump B</t>
         </is>
@@ -4831,7 +4870,7 @@
           <t>PS5-25-04</t>
         </is>
       </c>
-      <c r="B137" s="36" t="inlineStr">
+      <c r="B137" s="37" t="inlineStr">
         <is>
           <t>PS5-25-04 - Crude Oil Export Pump C</t>
         </is>
@@ -4859,7 +4898,7 @@
           <t>PS5-25-05</t>
         </is>
       </c>
-      <c r="B138" s="36" t="inlineStr">
+      <c r="B138" s="37" t="inlineStr">
         <is>
           <t>PS5-25-05 - Crude Oil Export Pumps Bypass</t>
         </is>
@@ -4887,7 +4926,7 @@
           <t>PS5-25-06</t>
         </is>
       </c>
-      <c r="B139" s="36" t="inlineStr">
+      <c r="B139" s="37" t="inlineStr">
         <is>
           <t>PS5-25-06 - Crude Oil Export Pumps Discharge</t>
         </is>
@@ -4915,7 +4954,7 @@
           <t>PS5-25-07</t>
         </is>
       </c>
-      <c r="B140" s="36" t="inlineStr">
+      <c r="B140" s="37" t="inlineStr">
         <is>
           <t>PS5-25-07 - Export Pipeline Pig Launcher</t>
         </is>
@@ -4943,7 +4982,7 @@
           <t>PS5-28-01</t>
         </is>
       </c>
-      <c r="B141" s="36" t="inlineStr">
+      <c r="B141" s="37" t="inlineStr">
         <is>
           <t>PS5-28-01 - Closed Drain Header 1</t>
         </is>
@@ -4971,7 +5010,7 @@
           <t>PS5-28-02</t>
         </is>
       </c>
-      <c r="B142" s="36" t="inlineStr">
+      <c r="B142" s="37" t="inlineStr">
         <is>
           <t>PS5-28-02 - Closed Drain Header 2</t>
         </is>
@@ -4999,7 +5038,7 @@
           <t>PS5-28-03</t>
         </is>
       </c>
-      <c r="B143" s="36" t="inlineStr">
+      <c r="B143" s="37" t="inlineStr">
         <is>
           <t>PS5-28-03 - Closed Drain Drum and Pump 01</t>
         </is>
@@ -5027,7 +5066,7 @@
           <t>PS5-28-04</t>
         </is>
       </c>
-      <c r="B144" s="36" t="inlineStr">
+      <c r="B144" s="37" t="inlineStr">
         <is>
           <t>PS5-28-04 - Closed Drain Drum and Pump 02</t>
         </is>
@@ -5055,7 +5094,7 @@
           <t>PS5-28-05</t>
         </is>
       </c>
-      <c r="B145" s="36" t="inlineStr">
+      <c r="B145" s="37" t="inlineStr">
         <is>
           <t>PS5-28-05 - HP Relief Header</t>
         </is>
@@ -5083,7 +5122,7 @@
           <t>PS5-28-06</t>
         </is>
       </c>
-      <c r="B146" s="36" t="inlineStr">
+      <c r="B146" s="37" t="inlineStr">
         <is>
           <t>PS5-28-06 - Relief Drum and Pump</t>
         </is>
@@ -5111,7 +5150,7 @@
           <t>PS5-28-07</t>
         </is>
       </c>
-      <c r="B147" s="36" t="inlineStr">
+      <c r="B147" s="37" t="inlineStr">
         <is>
           <t>PS5-28-07 - Open Drains (OD2)</t>
         </is>
@@ -5139,7 +5178,7 @@
           <t>PS5-28-08</t>
         </is>
       </c>
-      <c r="B148" s="36" t="inlineStr">
+      <c r="B148" s="37" t="inlineStr">
         <is>
           <t>PS5-28-08 - Open Drain Sump and Pumps</t>
         </is>
@@ -5167,7 +5206,7 @@
           <t>PS5-28-09</t>
         </is>
       </c>
-      <c r="B149" s="36" t="inlineStr">
+      <c r="B149" s="37" t="inlineStr">
         <is>
           <t>PS5-28-09 - Observation Basin</t>
         </is>
@@ -5195,7 +5234,7 @@
           <t>PS5-28-10</t>
         </is>
       </c>
-      <c r="B150" s="36" t="inlineStr">
+      <c r="B150" s="37" t="inlineStr">
         <is>
           <t>PS5-28-10 - Oil Skimmer Package</t>
         </is>
@@ -5223,7 +5262,7 @@
           <t>PS5-28-11</t>
         </is>
       </c>
-      <c r="B151" s="36" t="inlineStr">
+      <c r="B151" s="37" t="inlineStr">
         <is>
           <t>PS5-28-11 - Open Drain Interceptor</t>
         </is>
@@ -5251,7 +5290,7 @@
           <t>PS5-28-12</t>
         </is>
       </c>
-      <c r="B152" s="36" t="inlineStr">
+      <c r="B152" s="37" t="inlineStr">
         <is>
           <t>PS5-28-12 - Open Drains (OD3)</t>
         </is>
@@ -5279,7 +5318,7 @@
           <t>PS5-28-13</t>
         </is>
       </c>
-      <c r="B153" s="36" t="inlineStr">
+      <c r="B153" s="37" t="inlineStr">
         <is>
           <t>PS5-28-13 - Seal Oil Drain Drum &amp; Pump A</t>
         </is>
@@ -5307,7 +5346,7 @@
           <t>PS5-28-14</t>
         </is>
       </c>
-      <c r="B154" s="36" t="inlineStr">
+      <c r="B154" s="37" t="inlineStr">
         <is>
           <t>PS5-28-14 - Seal Oil Drain Drum &amp; Pump B</t>
         </is>
@@ -5335,7 +5374,7 @@
           <t>PS5-28-15</t>
         </is>
       </c>
-      <c r="B155" s="36" t="inlineStr">
+      <c r="B155" s="37" t="inlineStr">
         <is>
           <t>PS5-28-15 - Seal Oil Drain Drum &amp; Pump C</t>
         </is>
@@ -5363,7 +5402,7 @@
           <t>PS5-28-16</t>
         </is>
       </c>
-      <c r="B156" s="36" t="inlineStr">
+      <c r="B156" s="37" t="inlineStr">
         <is>
           <t>PS5-28-16 - LP Relief Header</t>
         </is>
@@ -5391,7 +5430,7 @@
           <t>PS5-28-17</t>
         </is>
       </c>
-      <c r="B157" s="36" t="inlineStr">
+      <c r="B157" s="37" t="inlineStr">
         <is>
           <t>PS5-28-17 - Reinjection Pump</t>
         </is>
@@ -5419,7 +5458,7 @@
           <t>PS5-50-01</t>
         </is>
       </c>
-      <c r="B158" s="36" t="inlineStr">
+      <c r="B158" s="37" t="inlineStr">
         <is>
           <t>PS5-50-01 - Water Well Submersible Pumps (3100)</t>
         </is>
@@ -5447,7 +5486,7 @@
           <t>PS5-50-02</t>
         </is>
       </c>
-      <c r="B159" s="36" t="inlineStr">
+      <c r="B159" s="37" t="inlineStr">
         <is>
           <t>PS5-50-02 - Water Well Submersible Pumps (3200)</t>
         </is>
@@ -5475,7 +5514,7 @@
           <t>PS5-50-03</t>
         </is>
       </c>
-      <c r="B160" s="36" t="inlineStr">
+      <c r="B160" s="37" t="inlineStr">
         <is>
           <t>PS5-50-03 - Water Pre-Treatment Package</t>
         </is>
@@ -5503,7 +5542,7 @@
           <t>PS5-53-01</t>
         </is>
       </c>
-      <c r="B161" s="36" t="inlineStr">
+      <c r="B161" s="37" t="inlineStr">
         <is>
           <t>PS5-53-01 - Utility Water / Storage Tank</t>
         </is>
@@ -5531,7 +5570,7 @@
           <t>PS5-53-02</t>
         </is>
       </c>
-      <c r="B162" s="36" t="inlineStr">
+      <c r="B162" s="37" t="inlineStr">
         <is>
           <t>PS5-53-02 - Water Distribution Pump A/B</t>
         </is>
@@ -5559,7 +5598,7 @@
           <t>PS5-53-03</t>
         </is>
       </c>
-      <c r="B163" s="36" t="inlineStr">
+      <c r="B163" s="37" t="inlineStr">
         <is>
           <t>PS5-53-03 - Water Softener Package</t>
         </is>
@@ -5587,7 +5626,7 @@
           <t>PS5-53-04</t>
         </is>
       </c>
-      <c r="B164" s="36" t="inlineStr">
+      <c r="B164" s="37" t="inlineStr">
         <is>
           <t>PS5-53-04 - Water Treatment Purification Package</t>
         </is>
@@ -5615,7 +5654,7 @@
           <t>PS5-53-05</t>
         </is>
       </c>
-      <c r="B165" s="36" t="inlineStr">
+      <c r="B165" s="37" t="inlineStr">
         <is>
           <t>PS5-53-05 - Water Distribution Header</t>
         </is>
@@ -5643,7 +5682,7 @@
           <t>PS5-53-06</t>
         </is>
       </c>
-      <c r="B166" s="36" t="inlineStr">
+      <c r="B166" s="37" t="inlineStr">
         <is>
           <t>PS5-53-06 - Water Distribution Consumers</t>
         </is>
@@ -5671,7 +5710,7 @@
           <t>PS5-60-01</t>
         </is>
       </c>
-      <c r="B167" s="36" t="inlineStr">
+      <c r="B167" s="37" t="inlineStr">
         <is>
           <t>PS5-60-01 - Power Generation Package A</t>
         </is>
@@ -5699,7 +5738,7 @@
           <t>PS5-60-02</t>
         </is>
       </c>
-      <c r="B168" s="36" t="inlineStr">
+      <c r="B168" s="37" t="inlineStr">
         <is>
           <t>PS5-60-02 - Power Gen Package A (UCP)</t>
         </is>
@@ -5727,7 +5766,7 @@
           <t>PS5-60-03</t>
         </is>
       </c>
-      <c r="B169" s="36" t="inlineStr">
+      <c r="B169" s="37" t="inlineStr">
         <is>
           <t>PS5-60-03 - Power Gen Package A Generator Auxiliary MCCs &amp; DBs</t>
         </is>
@@ -5755,7 +5794,7 @@
           <t>PS5-60-04</t>
         </is>
       </c>
-      <c r="B170" s="36" t="inlineStr">
+      <c r="B170" s="37" t="inlineStr">
         <is>
           <t>PS5-60-04 - Power Generation Package B</t>
         </is>
@@ -5783,7 +5822,7 @@
           <t>PS5-60-05</t>
         </is>
       </c>
-      <c r="B171" s="36" t="inlineStr">
+      <c r="B171" s="37" t="inlineStr">
         <is>
           <t>PS5-60-05 - Power Gen Package B (UCP)</t>
         </is>
@@ -5811,7 +5850,7 @@
           <t>PS5-60-06</t>
         </is>
       </c>
-      <c r="B172" s="36" t="inlineStr">
+      <c r="B172" s="37" t="inlineStr">
         <is>
           <t>PS5-60-06 - Power Gen Package B Generator Auxiliary MCCs &amp; DBs</t>
         </is>
@@ -5839,7 +5878,7 @@
           <t>PS5-60-07</t>
         </is>
       </c>
-      <c r="B173" s="36" t="inlineStr">
+      <c r="B173" s="37" t="inlineStr">
         <is>
           <t>PS5-60-07 - Power Generation Package C</t>
         </is>
@@ -5867,7 +5906,7 @@
           <t>PS5-60-08</t>
         </is>
       </c>
-      <c r="B174" s="36" t="inlineStr">
+      <c r="B174" s="37" t="inlineStr">
         <is>
           <t>PS5-60-08 - Power Gen Package C (UCP)</t>
         </is>
@@ -5895,7 +5934,7 @@
           <t>PS5-60-09</t>
         </is>
       </c>
-      <c r="B175" s="36" t="inlineStr">
+      <c r="B175" s="37" t="inlineStr">
         <is>
           <t>PS5-60-09 - Power Gen Package C Generator Auxiliary MCCs &amp; DBs</t>
         </is>
@@ -5923,7 +5962,7 @@
           <t>PS5-60-10</t>
         </is>
       </c>
-      <c r="B176" s="36" t="inlineStr">
+      <c r="B176" s="37" t="inlineStr">
         <is>
           <t>PS5-60-10 - Power Generation Package D</t>
         </is>
@@ -5951,7 +5990,7 @@
           <t>PS5-60-11</t>
         </is>
       </c>
-      <c r="B177" s="36" t="inlineStr">
+      <c r="B177" s="37" t="inlineStr">
         <is>
           <t>PS5-60-11 - Power Gen Package D (UCP)</t>
         </is>
@@ -5979,7 +6018,7 @@
           <t>PS5-60-12</t>
         </is>
       </c>
-      <c r="B178" s="36" t="inlineStr">
+      <c r="B178" s="37" t="inlineStr">
         <is>
           <t>PS5-60-12 - Power Gen Package D Generator Auxiliary MCCs &amp; DBs</t>
         </is>
@@ -6007,7 +6046,7 @@
           <t>PS5-60-13</t>
         </is>
       </c>
-      <c r="B179" s="36" t="inlineStr">
+      <c r="B179" s="37" t="inlineStr">
         <is>
           <t>PS5-60-13 - Power Generation Package E</t>
         </is>
@@ -6035,7 +6074,7 @@
           <t>PS5-60-14</t>
         </is>
       </c>
-      <c r="B180" s="36" t="inlineStr">
+      <c r="B180" s="37" t="inlineStr">
         <is>
           <t>PS5-60-14 - Power Gen Package E (UCP)</t>
         </is>
@@ -6063,7 +6102,7 @@
           <t>PS5-60-15</t>
         </is>
       </c>
-      <c r="B181" s="36" t="inlineStr">
+      <c r="B181" s="37" t="inlineStr">
         <is>
           <t>PS5-60-15 - Power Gen Package E Generator Auxiliary MCCs &amp; DBs</t>
         </is>
@@ -6091,7 +6130,7 @@
           <t>PS5-60-16</t>
         </is>
       </c>
-      <c r="B182" s="36" t="inlineStr">
+      <c r="B182" s="37" t="inlineStr">
         <is>
           <t>PS5-60-16 - Power Generation Package F</t>
         </is>
@@ -6119,7 +6158,7 @@
           <t>PS5-60-17</t>
         </is>
       </c>
-      <c r="B183" s="36" t="inlineStr">
+      <c r="B183" s="37" t="inlineStr">
         <is>
           <t>PS5-60-17 - Power Gen Package F (UCP)</t>
         </is>
@@ -6147,7 +6186,7 @@
           <t>PS5-60-18</t>
         </is>
       </c>
-      <c r="B184" s="36" t="inlineStr">
+      <c r="B184" s="37" t="inlineStr">
         <is>
           <t>PS5-60-18 - Power Gen Package F Generator Auxiliary MCCs &amp; DBs</t>
         </is>
@@ -6175,7 +6214,7 @@
           <t>PS5-60-19</t>
         </is>
       </c>
-      <c r="B185" s="36" t="inlineStr">
+      <c r="B185" s="37" t="inlineStr">
         <is>
           <t>PS5-60-19 - Power Generation Package G</t>
         </is>
@@ -6203,7 +6242,7 @@
           <t>PS5-60-20</t>
         </is>
       </c>
-      <c r="B186" s="36" t="inlineStr">
+      <c r="B186" s="37" t="inlineStr">
         <is>
           <t>PS5-60-20 - Power Gen Package G (UCP)</t>
         </is>
@@ -6231,7 +6270,7 @@
           <t>PS5-60-21</t>
         </is>
       </c>
-      <c r="B187" s="36" t="inlineStr">
+      <c r="B187" s="37" t="inlineStr">
         <is>
           <t>PS5-60-21 - Power Gen Package G Generator Auxiliary MCCs &amp; DBs</t>
         </is>
@@ -6259,7 +6298,7 @@
           <t>PS5-60-22</t>
         </is>
       </c>
-      <c r="B188" s="36" t="inlineStr">
+      <c r="B188" s="37" t="inlineStr">
         <is>
           <t>PS5-60-22 - Power Gen Master UCP</t>
         </is>
@@ -6287,7 +6326,7 @@
           <t>PS5-60-23</t>
         </is>
       </c>
-      <c r="B189" s="36" t="inlineStr">
+      <c r="B189" s="37" t="inlineStr">
         <is>
           <t>PS5-60-23 - Instrument Air Distribution lines</t>
         </is>
@@ -6315,7 +6354,7 @@
           <t>PS5-60-24</t>
         </is>
       </c>
-      <c r="B190" s="36" t="inlineStr">
+      <c r="B190" s="37" t="inlineStr">
         <is>
           <t>PS5-60-24 - Cooling Water Tank &amp; Pump</t>
         </is>
@@ -6343,7 +6382,7 @@
           <t>PS5-60-25</t>
         </is>
       </c>
-      <c r="B191" s="36" t="inlineStr">
+      <c r="B191" s="37" t="inlineStr">
         <is>
           <t>PS5-60-25 - Cooling Water Maintenance Tank &amp; Return Pump</t>
         </is>
@@ -6371,7 +6410,7 @@
           <t>PS5-60-26</t>
         </is>
       </c>
-      <c r="B192" s="36" t="inlineStr">
+      <c r="B192" s="37" t="inlineStr">
         <is>
           <t>PS5-60-26 - Instrument Air Compressor Skid</t>
         </is>
@@ -6399,7 +6438,7 @@
           <t>PS5-60-27</t>
         </is>
       </c>
-      <c r="B193" s="36" t="inlineStr">
+      <c r="B193" s="37" t="inlineStr">
         <is>
           <t>PS5-60-27 - Compressed Air Starting Skid</t>
         </is>
@@ -6427,7 +6466,7 @@
           <t>PS5-60-28</t>
         </is>
       </c>
-      <c r="B194" s="36" t="inlineStr">
+      <c r="B194" s="37" t="inlineStr">
         <is>
           <t>PS5-60-28 - Air Receiver A &amp; Air Regulator A</t>
         </is>
@@ -6455,7 +6494,7 @@
           <t>PS5-60-29</t>
         </is>
       </c>
-      <c r="B195" s="36" t="inlineStr">
+      <c r="B195" s="37" t="inlineStr">
         <is>
           <t>PS5-60-29 - Air Receiver B &amp; Air Regulator B</t>
         </is>
@@ -6483,7 +6522,7 @@
           <t>PS5-60-30</t>
         </is>
       </c>
-      <c r="B196" s="36" t="inlineStr">
+      <c r="B196" s="37" t="inlineStr">
         <is>
           <t>PS5-60-30 - Air Receiver C &amp; Air Regulator C</t>
         </is>
@@ -6511,7 +6550,7 @@
           <t>PS5-60-31</t>
         </is>
       </c>
-      <c r="B197" s="36" t="inlineStr">
+      <c r="B197" s="37" t="inlineStr">
         <is>
           <t>PS5-60-31 - Air Receiver D &amp; Air Regulator D</t>
         </is>
@@ -6539,7 +6578,7 @@
           <t>PS5-60-32</t>
         </is>
       </c>
-      <c r="B198" s="36" t="inlineStr">
+      <c r="B198" s="37" t="inlineStr">
         <is>
           <t>PS5-60-32 - Air Receiver E &amp; Air Regulator E</t>
         </is>
@@ -6567,7 +6606,7 @@
           <t>PS5-60-33</t>
         </is>
       </c>
-      <c r="B199" s="36" t="inlineStr">
+      <c r="B199" s="37" t="inlineStr">
         <is>
           <t>PS5-60-33 - Air Receiver F &amp; Air Regulator F</t>
         </is>
@@ -6595,7 +6634,7 @@
           <t>PS5-60-34</t>
         </is>
       </c>
-      <c r="B200" s="36" t="inlineStr">
+      <c r="B200" s="37" t="inlineStr">
         <is>
           <t>PS5-60-34 - Air Receiver G &amp; Air Regulator G</t>
         </is>
@@ -6623,7 +6662,7 @@
           <t>PS5-60-35</t>
         </is>
       </c>
-      <c r="B201" s="36" t="inlineStr">
+      <c r="B201" s="37" t="inlineStr">
         <is>
           <t>PS5-60-35 - Injector Tip Cooling Module A</t>
         </is>
@@ -6651,7 +6690,7 @@
           <t>PS5-60-36</t>
         </is>
       </c>
-      <c r="B202" s="36" t="inlineStr">
+      <c r="B202" s="37" t="inlineStr">
         <is>
           <t>PS5-60-36 - Injector Tip Cooling Module B</t>
         </is>
@@ -6679,7 +6718,7 @@
           <t>PS5-60-37</t>
         </is>
       </c>
-      <c r="B203" s="36" t="inlineStr">
+      <c r="B203" s="37" t="inlineStr">
         <is>
           <t>PS5-60-37 - Injector Tip Cooling Module C</t>
         </is>
@@ -6707,7 +6746,7 @@
           <t>PS5-60-38</t>
         </is>
       </c>
-      <c r="B204" s="36" t="inlineStr">
+      <c r="B204" s="37" t="inlineStr">
         <is>
           <t>PS5-60-38 - Injector Tip Cooling Module D</t>
         </is>
@@ -6735,7 +6774,7 @@
           <t>PS5-60-39</t>
         </is>
       </c>
-      <c r="B205" s="36" t="inlineStr">
+      <c r="B205" s="37" t="inlineStr">
         <is>
           <t>PS5-60-39 - Injector Tip Cooling Module E</t>
         </is>
@@ -6763,7 +6802,7 @@
           <t>PS5-60-40</t>
         </is>
       </c>
-      <c r="B206" s="36" t="inlineStr">
+      <c r="B206" s="37" t="inlineStr">
         <is>
           <t>PS5-60-40 - Injector Tip Cooling Module F</t>
         </is>
@@ -6791,7 +6830,7 @@
           <t>PS5-60-41</t>
         </is>
       </c>
-      <c r="B207" s="36" t="inlineStr">
+      <c r="B207" s="37" t="inlineStr">
         <is>
           <t>PS5-60-41 - Injector Tip Cooling Module G</t>
         </is>
@@ -6819,7 +6858,7 @@
           <t>PS5-60-42</t>
         </is>
       </c>
-      <c r="B208" s="36" t="inlineStr">
+      <c r="B208" s="37" t="inlineStr">
         <is>
           <t>PS5-60-42 - Oil Mist Separator Skid PS5-60-VS-9100A</t>
         </is>
@@ -6847,7 +6886,7 @@
           <t>PS5-60-43</t>
         </is>
       </c>
-      <c r="B209" s="36" t="inlineStr">
+      <c r="B209" s="37" t="inlineStr">
         <is>
           <t>PS5-60-43 - Oil Mist Separator Skid PS5-60-VS-9100B</t>
         </is>
@@ -6875,7 +6914,7 @@
           <t>PS5-60-44</t>
         </is>
       </c>
-      <c r="B210" s="36" t="inlineStr">
+      <c r="B210" s="37" t="inlineStr">
         <is>
           <t>PS5-60-44 - Oil Mist Separator Skid PS5-60-VS-9100C</t>
         </is>
@@ -6903,7 +6942,7 @@
           <t>PS5-60-45</t>
         </is>
       </c>
-      <c r="B211" s="36" t="inlineStr">
+      <c r="B211" s="37" t="inlineStr">
         <is>
           <t>PS5-60-45 - Oil Mist Separator Skid PS5-60-VS-9100D</t>
         </is>
@@ -6931,7 +6970,7 @@
           <t>PS5-60-46</t>
         </is>
       </c>
-      <c r="B212" s="36" t="inlineStr">
+      <c r="B212" s="37" t="inlineStr">
         <is>
           <t>PS5-60-46 - Oil Mist Separator Skid PS5-60-VS-9100E</t>
         </is>
@@ -6959,7 +6998,7 @@
           <t>PS5-60-47</t>
         </is>
       </c>
-      <c r="B213" s="36" t="inlineStr">
+      <c r="B213" s="37" t="inlineStr">
         <is>
           <t>PS5-60-47 - Oil Mist Separator Skid PS5-60-VS-9100F</t>
         </is>
@@ -6987,7 +7026,7 @@
           <t>PS5-60-48</t>
         </is>
       </c>
-      <c r="B214" s="36" t="inlineStr">
+      <c r="B214" s="37" t="inlineStr">
         <is>
           <t>PS5-60-48 - Oil Mist Separator Skid PS5-60-VS-9100G</t>
         </is>
@@ -7015,7 +7054,7 @@
           <t>PS5-60-49</t>
         </is>
       </c>
-      <c r="B215" s="36" t="inlineStr">
+      <c r="B215" s="37" t="inlineStr">
         <is>
           <t>PS5-60-49 - Lube Oil Separator Module PS5-60-UO-81100A</t>
         </is>
@@ -7043,7 +7082,7 @@
           <t>PS5-60-50</t>
         </is>
       </c>
-      <c r="B216" s="36" t="inlineStr">
+      <c r="B216" s="37" t="inlineStr">
         <is>
           <t>PS5-60-50 - Lube Oil Separator Module PS5-60-UO-81100B</t>
         </is>
@@ -7071,7 +7110,7 @@
           <t>PS5-60-51</t>
         </is>
       </c>
-      <c r="B217" s="36" t="inlineStr">
+      <c r="B217" s="37" t="inlineStr">
         <is>
           <t>PS5-60-51 - Lube Oil Separator Module PS5-60-UO-81100C</t>
         </is>
@@ -7099,7 +7138,7 @@
           <t>PS5-60-52</t>
         </is>
       </c>
-      <c r="B218" s="36" t="inlineStr">
+      <c r="B218" s="37" t="inlineStr">
         <is>
           <t>PS5-60-52 - Lube Oil Separator Module PS5-60-UO-81100D</t>
         </is>
@@ -7127,7 +7166,7 @@
           <t>PS5-60-53</t>
         </is>
       </c>
-      <c r="B219" s="36" t="inlineStr">
+      <c r="B219" s="37" t="inlineStr">
         <is>
           <t>PS5-60-53 - Lube Oil Separator Module PS5-60-UO-81100E</t>
         </is>
@@ -7155,7 +7194,7 @@
           <t>PS5-60-54</t>
         </is>
       </c>
-      <c r="B220" s="36" t="inlineStr">
+      <c r="B220" s="37" t="inlineStr">
         <is>
           <t>PS5-60-54 - Lube Oil Separator Module PS5-60-UO-81100F</t>
         </is>
@@ -7183,7 +7222,7 @@
           <t>PS5-60-55</t>
         </is>
       </c>
-      <c r="B221" s="36" t="inlineStr">
+      <c r="B221" s="37" t="inlineStr">
         <is>
           <t>PS5-60-55 - Lube Oil Separator Module PS5-60-UO-81100G</t>
         </is>
@@ -7211,7 +7250,7 @@
           <t>PS5-60-56</t>
         </is>
       </c>
-      <c r="B222" s="36" t="inlineStr">
+      <c r="B222" s="37" t="inlineStr">
         <is>
           <t>PS5-60-56 - Fuel Conditioning Module PS5-60-UZ-8900A</t>
         </is>
@@ -7239,7 +7278,7 @@
           <t>PS5-60-57</t>
         </is>
       </c>
-      <c r="B223" s="36" t="inlineStr">
+      <c r="B223" s="37" t="inlineStr">
         <is>
           <t>PS5-60-57 - Fuel Conditioning Module PS5-60-UZ-8900A (UCP)</t>
         </is>
@@ -7267,7 +7306,7 @@
           <t>PS5-60-58</t>
         </is>
       </c>
-      <c r="B224" s="36" t="inlineStr">
+      <c r="B224" s="37" t="inlineStr">
         <is>
           <t>PS5-60-58 - Fuel Conditioning Module PS5-60-UZ-8900B</t>
         </is>
@@ -7295,7 +7334,7 @@
           <t>PS5-60-59</t>
         </is>
       </c>
-      <c r="B225" s="36" t="inlineStr">
+      <c r="B225" s="37" t="inlineStr">
         <is>
           <t>PS5-60-59 - Fuel Conditioning Module PS5-60-UZ-8900B (UCP)</t>
         </is>
@@ -7323,7 +7362,7 @@
           <t>PS5-60-60</t>
         </is>
       </c>
-      <c r="B226" s="36" t="inlineStr">
+      <c r="B226" s="37" t="inlineStr">
         <is>
           <t>PS5-60-60 - Fuel Conditioning Module PS5-60-UZ-8900C</t>
         </is>
@@ -7351,7 +7390,7 @@
           <t>PS5-60-61</t>
         </is>
       </c>
-      <c r="B227" s="36" t="inlineStr">
+      <c r="B227" s="37" t="inlineStr">
         <is>
           <t>PS5-60-61 - Fuel Conditioning Module PS5-60-UZ-8900C (UCP)</t>
         </is>
@@ -7379,7 +7418,7 @@
           <t>PS5-60-62</t>
         </is>
       </c>
-      <c r="B228" s="36" t="inlineStr">
+      <c r="B228" s="37" t="inlineStr">
         <is>
           <t>PS5-60-62 - Fuel Conditioning Module PS5-60-UZ-8900D</t>
         </is>
@@ -7407,7 +7446,7 @@
           <t>PS5-60-63</t>
         </is>
       </c>
-      <c r="B229" s="36" t="inlineStr">
+      <c r="B229" s="37" t="inlineStr">
         <is>
           <t>PS5-60-63 - Fuel Conditioning Module PS5-60-UZ-8900D (UCP)</t>
         </is>
@@ -7435,7 +7474,7 @@
           <t>PS5-60-64</t>
         </is>
       </c>
-      <c r="B230" s="36" t="inlineStr">
+      <c r="B230" s="37" t="inlineStr">
         <is>
           <t>PS5-60-64 - Fuel Conditioning Module PS5-60-UZ-8900E</t>
         </is>
@@ -7463,7 +7502,7 @@
           <t>PS5-60-65</t>
         </is>
       </c>
-      <c r="B231" s="36" t="inlineStr">
+      <c r="B231" s="37" t="inlineStr">
         <is>
           <t>PS5-60-65 - Fuel Conditioning Module PS5-60-UZ-8900E (UCP)</t>
         </is>
@@ -7491,7 +7530,7 @@
           <t>PS5-60-66</t>
         </is>
       </c>
-      <c r="B232" s="36" t="inlineStr">
+      <c r="B232" s="37" t="inlineStr">
         <is>
           <t>PS5-60-66 - Fuel Conditioning Module PS5-60-UZ-8900F</t>
         </is>
@@ -7519,7 +7558,7 @@
           <t>PS5-60-67</t>
         </is>
       </c>
-      <c r="B233" s="36" t="inlineStr">
+      <c r="B233" s="37" t="inlineStr">
         <is>
           <t>PS5-60-67 - Fuel Conditioning Module PS5-60-UZ-8900F (UCP)</t>
         </is>
@@ -7547,7 +7586,7 @@
           <t>PS5-60-68</t>
         </is>
       </c>
-      <c r="B234" s="36" t="inlineStr">
+      <c r="B234" s="37" t="inlineStr">
         <is>
           <t>PS5-60-68 - Fuel Conditioning Module PS5-60-UZ-8900G</t>
         </is>
@@ -7575,7 +7614,7 @@
           <t>PS5-60-69</t>
         </is>
       </c>
-      <c r="B235" s="36" t="inlineStr">
+      <c r="B235" s="37" t="inlineStr">
         <is>
           <t>PS5-60-69 - Fuel Conditioning Module PS5-60-UZ-8900G (UCP)</t>
         </is>
@@ -7603,7 +7642,7 @@
           <t>PS5-60-70</t>
         </is>
       </c>
-      <c r="B236" s="36" t="inlineStr">
+      <c r="B236" s="37" t="inlineStr">
         <is>
           <t>PS5-60-70 - Engine A Cooling system</t>
         </is>
@@ -7631,7 +7670,7 @@
           <t>PS5-60-71</t>
         </is>
       </c>
-      <c r="B237" s="36" t="inlineStr">
+      <c r="B237" s="37" t="inlineStr">
         <is>
           <t>PS5-60-71 - Engine B Cooling system</t>
         </is>
@@ -7659,7 +7698,7 @@
           <t>PS5-60-72</t>
         </is>
       </c>
-      <c r="B238" s="36" t="inlineStr">
+      <c r="B238" s="37" t="inlineStr">
         <is>
           <t>PS5-60-72 - Engine C Cooling system</t>
         </is>
@@ -7687,7 +7726,7 @@
           <t>PS5-60-73</t>
         </is>
       </c>
-      <c r="B239" s="36" t="inlineStr">
+      <c r="B239" s="37" t="inlineStr">
         <is>
           <t>PS5-60-73 - Engine D Cooling system</t>
         </is>
@@ -7715,7 +7754,7 @@
           <t>PS5-60-74</t>
         </is>
       </c>
-      <c r="B240" s="36" t="inlineStr">
+      <c r="B240" s="37" t="inlineStr">
         <is>
           <t>PS5-60-74 - Engine E Cooling system</t>
         </is>
@@ -7743,7 +7782,7 @@
           <t>PS5-60-75</t>
         </is>
       </c>
-      <c r="B241" s="36" t="inlineStr">
+      <c r="B241" s="37" t="inlineStr">
         <is>
           <t>PS5-60-75 - Engine F Cooling system</t>
         </is>
@@ -7771,7 +7810,7 @@
           <t>PS5-60-76</t>
         </is>
       </c>
-      <c r="B242" s="36" t="inlineStr">
+      <c r="B242" s="37" t="inlineStr">
         <is>
           <t>PS5-60-76 - Engine G Cooling system</t>
         </is>
@@ -7799,7 +7838,7 @@
           <t>PS5-61-01</t>
         </is>
       </c>
-      <c r="B243" s="36" t="inlineStr">
+      <c r="B243" s="37" t="inlineStr">
         <is>
           <t>PS5-61-01 - 33kV Switchboard EITS Building (PS5-61-IJ-0001)</t>
         </is>
@@ -7827,7 +7866,7 @@
           <t>PS5-61-02</t>
         </is>
       </c>
-      <c r="B244" s="36" t="inlineStr">
+      <c r="B244" s="37" t="inlineStr">
         <is>
           <t>PS5-61-02 - 6.6kV Switchboard and Transformer LLHT North - EITS Building (PS5-61-IJ-0010)</t>
         </is>
@@ -7855,7 +7894,7 @@
           <t>PS5-61-03</t>
         </is>
       </c>
-      <c r="B245" s="36" t="inlineStr">
+      <c r="B245" s="37" t="inlineStr">
         <is>
           <t>PS5-61-03 - 6.6kV Switchboard and Transformer LLHT South - EITS Building (PS5-61-IJ-0011)</t>
         </is>
@@ -7883,7 +7922,7 @@
           <t>PS5-61-04</t>
         </is>
       </c>
-      <c r="B246" s="36" t="inlineStr">
+      <c r="B246" s="37" t="inlineStr">
         <is>
           <t>PS5-61-04 - 0.4kV Switchboard Office &amp; Facilities Building (PS5-61-IK-0005)</t>
         </is>
@@ -7911,7 +7950,7 @@
           <t>PS5-61-05</t>
         </is>
       </c>
-      <c r="B247" s="36" t="inlineStr">
+      <c r="B247" s="37" t="inlineStr">
         <is>
           <t>PS5-61-05 - 0.4kV Switchboard Power Generator Building (PS5-61-IK-0003)</t>
         </is>
@@ -7939,7 +7978,7 @@
           <t>PS5-61-06</t>
         </is>
       </c>
-      <c r="B248" s="36" t="inlineStr">
+      <c r="B248" s="37" t="inlineStr">
         <is>
           <t>PS5-61-06 - 0.4kV Switchboard Power Generator Building (PS5-61-IK-0006)</t>
         </is>
@@ -7967,7 +8006,7 @@
           <t>PS5-61-07</t>
         </is>
       </c>
-      <c r="B249" s="36" t="inlineStr">
+      <c r="B249" s="37" t="inlineStr">
         <is>
           <t>PS5-61-07 - 0.4kV Switchboard EITS Building (PS5-61-IK-0001)</t>
         </is>
@@ -7995,7 +8034,7 @@
           <t>PS5-61-08</t>
         </is>
       </c>
-      <c r="B250" s="36" t="inlineStr">
+      <c r="B250" s="37" t="inlineStr">
         <is>
           <t>PS5-61-08 - Electrical Control System</t>
         </is>
@@ -8023,7 +8062,7 @@
           <t>PS5-61-09</t>
         </is>
       </c>
-      <c r="B251" s="36" t="inlineStr">
+      <c r="B251" s="37" t="inlineStr">
         <is>
           <t>PS5-61-09 - Outdoor Power Distribution Board - PS5-61-IG-0014</t>
         </is>
@@ -8051,7 +8090,7 @@
           <t>PS5-61-10</t>
         </is>
       </c>
-      <c r="B252" s="36" t="inlineStr">
+      <c r="B252" s="37" t="inlineStr">
         <is>
           <t>PS5-61-10 - Outdoor Valves Distribution Board - PS5-61-IG-0042</t>
         </is>
@@ -8079,7 +8118,7 @@
           <t>PS5-61-11</t>
         </is>
       </c>
-      <c r="B253" s="36" t="inlineStr">
+      <c r="B253" s="37" t="inlineStr">
         <is>
           <t>PS5-61-11 - Outdoor Valves Distribution Board - PS5-61-IG-0043</t>
         </is>
@@ -8107,7 +8146,7 @@
           <t>PS5-61-12</t>
         </is>
       </c>
-      <c r="B254" s="36" t="inlineStr">
+      <c r="B254" s="37" t="inlineStr">
         <is>
           <t>PS5-61-12 - EITS 33kV Bld. Normal Auxiliary DP - PS5-61-IG-0008</t>
         </is>
@@ -8135,7 +8174,7 @@
           <t>PS5-61-13</t>
         </is>
       </c>
-      <c r="B255" s="36" t="inlineStr">
+      <c r="B255" s="37" t="inlineStr">
         <is>
           <t>PS5-61-13 - Power Distribution Board Office Building - PS5-61-IG-0020</t>
         </is>
@@ -8163,7 +8202,7 @@
           <t>PS5-61-14</t>
         </is>
       </c>
-      <c r="B256" s="36" t="inlineStr">
+      <c r="B256" s="37" t="inlineStr">
         <is>
           <t>PS5-61-14 - Power Distribution Board Workshop &amp; Warehouse - PS5-61-IG-0009</t>
         </is>
@@ -8191,7 +8230,7 @@
           <t>PS5-62-01</t>
         </is>
       </c>
-      <c r="B257" s="36" t="inlineStr">
+      <c r="B257" s="37" t="inlineStr">
         <is>
           <t>PS5-62-01 - Lighting Control Panel - PS5-62-IE-0001</t>
         </is>
@@ -8219,7 +8258,7 @@
           <t>PS5-62-02</t>
         </is>
       </c>
-      <c r="B258" s="36" t="inlineStr">
+      <c r="B258" s="37" t="inlineStr">
         <is>
           <t>PS5-62-02 - Lighting Control Panel - PS5-62-IE-0002</t>
         </is>
@@ -8247,7 +8286,7 @@
           <t>PS5-62-03</t>
         </is>
       </c>
-      <c r="B259" s="36" t="inlineStr">
+      <c r="B259" s="37" t="inlineStr">
         <is>
           <t>PS5-62-03 - Outdoor Emergency Lighting DB  - PS5-05-IG-0004</t>
         </is>
@@ -8275,7 +8314,7 @@
           <t>PS5-62-04</t>
         </is>
       </c>
-      <c r="B260" s="36" t="inlineStr">
+      <c r="B260" s="37" t="inlineStr">
         <is>
           <t>PS5-62-04 - Outdoor Emergency Lighting DB  - PS5-05-IG-0006</t>
         </is>
@@ -8303,7 +8342,7 @@
           <t>PS5-62-05</t>
         </is>
       </c>
-      <c r="B261" s="36" t="inlineStr">
+      <c r="B261" s="37" t="inlineStr">
         <is>
           <t>PS5-62-05 - Guard House Emergency L&amp;SP DB  - PS5-05-IG-0007</t>
         </is>
@@ -8331,7 +8370,7 @@
           <t>PS5-62-06</t>
         </is>
       </c>
-      <c r="B262" s="36" t="inlineStr">
+      <c r="B262" s="37" t="inlineStr">
         <is>
           <t>PS5-62-06 - CRO Generator Building Emergency Lighting DB  - PS5-05-IG-0025</t>
         </is>
@@ -8359,7 +8398,7 @@
           <t>PS5-62-07</t>
         </is>
       </c>
-      <c r="B263" s="36" t="inlineStr">
+      <c r="B263" s="37" t="inlineStr">
         <is>
           <t>PS5-62-07 - CRO Generator Electrical Building Emergency Lighting DB  - PS5-05-IG-0026</t>
         </is>
@@ -8387,7 +8426,7 @@
           <t>PS5-62-08</t>
         </is>
       </c>
-      <c r="B264" s="36" t="inlineStr">
+      <c r="B264" s="37" t="inlineStr">
         <is>
           <t>PS5-62-08 - Outdoor Normal Lighting  DB  - PS5-61-IG-0006</t>
         </is>
@@ -8415,7 +8454,7 @@
           <t>PS5-62-09</t>
         </is>
       </c>
-      <c r="B265" s="36" t="inlineStr">
+      <c r="B265" s="37" t="inlineStr">
         <is>
           <t>PS5-62-09 - Outdoor Normal Lighting DB  - PS5-61-IG-0007</t>
         </is>
@@ -8443,7 +8482,7 @@
           <t>PS5-62-10</t>
         </is>
       </c>
-      <c r="B266" s="36" t="inlineStr">
+      <c r="B266" s="37" t="inlineStr">
         <is>
           <t>PS5-62-10 - CRO Generator Building Normal L&amp;SP DB  - PS5-61-IG-0015</t>
         </is>
@@ -8471,7 +8510,7 @@
           <t>PS5-62-11</t>
         </is>
       </c>
-      <c r="B267" s="36" t="inlineStr">
+      <c r="B267" s="37" t="inlineStr">
         <is>
           <t>PS5-62-11 - CRO Generator Electrical Building Normal L&amp;SP DB  - PS5-61-IG-0016</t>
         </is>
@@ -8499,7 +8538,7 @@
           <t>PS5-62-12</t>
         </is>
       </c>
-      <c r="B268" s="36" t="inlineStr">
+      <c r="B268" s="37" t="inlineStr">
         <is>
           <t>PS5-62-12 - EITS 33kV Bld. Emergency L&amp;SP DP - PS5-05-IG-0003</t>
         </is>
@@ -8527,7 +8566,7 @@
           <t>PS5-62-13</t>
         </is>
       </c>
-      <c r="B269" s="36" t="inlineStr">
+      <c r="B269" s="37" t="inlineStr">
         <is>
           <t>PS5-62-13 - EITS 33kV Bld. Normal L&amp;SP DP - PS5-61-IG-0003</t>
         </is>
@@ -8555,7 +8594,7 @@
           <t>PS5-62-14</t>
         </is>
       </c>
-      <c r="B270" s="36" t="inlineStr">
+      <c r="B270" s="37" t="inlineStr">
         <is>
           <t>PS5-62-14 - Office Building Emergency L&amp;SP DB - PS5-05-IG-0002</t>
         </is>
@@ -8583,7 +8622,7 @@
           <t>PS5-62-15</t>
         </is>
       </c>
-      <c r="B271" s="36" t="inlineStr">
+      <c r="B271" s="37" t="inlineStr">
         <is>
           <t>PS5-62-15 - Office Building Normal L&amp;SP DB - PS5-61-IG-0002</t>
         </is>
@@ -8611,7 +8650,7 @@
           <t>PS5-62-16</t>
         </is>
       </c>
-      <c r="B272" s="36" t="inlineStr">
+      <c r="B272" s="37" t="inlineStr">
         <is>
           <t>PS5-62-16 - Guard Hut A Normal L&amp;SP DB - PS5-61-IG-0111</t>
         </is>
@@ -8639,7 +8678,7 @@
           <t>PS5-62-17</t>
         </is>
       </c>
-      <c r="B273" s="36" t="inlineStr">
+      <c r="B273" s="37" t="inlineStr">
         <is>
           <t>PS5-62-17 - Guard Hut B Normal L&amp;SP DB - PS5-61-IG-0112</t>
         </is>
@@ -8667,7 +8706,7 @@
           <t>PS5-62-18</t>
         </is>
       </c>
-      <c r="B274" s="36" t="inlineStr">
+      <c r="B274" s="37" t="inlineStr">
         <is>
           <t>PS5-62-18 - Workshop &amp; Warehouse Normal L&amp;SP DB - PS5-61-IG-0004</t>
         </is>
@@ -8695,7 +8734,7 @@
           <t>PS5-62-19</t>
         </is>
       </c>
-      <c r="B275" s="36" t="inlineStr">
+      <c r="B275" s="37" t="inlineStr">
         <is>
           <t>PS5-62-19 - Workshop &amp; Warehouse Emergency L&amp;SP DB - PS5-05-IG-0101</t>
         </is>
@@ -8723,7 +8762,7 @@
           <t>PS5-62-20</t>
         </is>
       </c>
-      <c r="B276" s="36" t="inlineStr">
+      <c r="B276" s="37" t="inlineStr">
         <is>
           <t>PS5-62-20 - Office Building Normal L&amp;SP DB - PS5-61-IG-0010</t>
         </is>
@@ -8751,7 +8790,7 @@
           <t>PS5-63-01</t>
         </is>
       </c>
-      <c r="B277" s="36" t="inlineStr">
+      <c r="B277" s="37" t="inlineStr">
         <is>
           <t>PS5-63-01 - Electrical Earthing</t>
         </is>
@@ -8779,7 +8818,7 @@
           <t>PS5-63-02</t>
         </is>
       </c>
-      <c r="B278" s="36" t="inlineStr">
+      <c r="B278" s="37" t="inlineStr">
         <is>
           <t>PS5-63-02 - Electrical Earthing - Office and Facilities building</t>
         </is>
@@ -8807,7 +8846,7 @@
           <t>PS5-63-03</t>
         </is>
       </c>
-      <c r="B279" s="36" t="inlineStr">
+      <c r="B279" s="37" t="inlineStr">
         <is>
           <t>PS5-63-03 - Electrical Earthing - Generator Building</t>
         </is>
@@ -8835,7 +8874,7 @@
           <t>PS5-63-04</t>
         </is>
       </c>
-      <c r="B280" s="36" t="inlineStr">
+      <c r="B280" s="37" t="inlineStr">
         <is>
           <t>PS5-63-04 - Electrical Earthing - EITS Building</t>
         </is>
@@ -8863,7 +8902,7 @@
           <t>PS5-63-05</t>
         </is>
       </c>
-      <c r="B281" s="36" t="inlineStr">
+      <c r="B281" s="37" t="inlineStr">
         <is>
           <t>PS5-63-05 - Electrical Earthing - Guard Hut A &amp; B</t>
         </is>
@@ -8891,7 +8930,7 @@
           <t>PS5-63-06</t>
         </is>
       </c>
-      <c r="B282" s="36" t="inlineStr">
+      <c r="B282" s="37" t="inlineStr">
         <is>
           <t>PS5-63-06 - Electrical Earthing - Guard House</t>
         </is>
@@ -8919,7 +8958,7 @@
           <t>PS5-63-07</t>
         </is>
       </c>
-      <c r="B283" s="36" t="inlineStr">
+      <c r="B283" s="37" t="inlineStr">
         <is>
           <t>PS5-63-07 - Electrical Earthing - Workshop &amp; Warehouse</t>
         </is>
@@ -8947,7 +8986,7 @@
           <t>PS5-71-01</t>
         </is>
       </c>
-      <c r="B284" s="36" t="inlineStr">
+      <c r="B284" s="37" t="inlineStr">
         <is>
           <t>PS5-71-01 - CFO Storage Tank Feed Heater</t>
         </is>
@@ -8975,7 +9014,7 @@
           <t>PS5-71-02</t>
         </is>
       </c>
-      <c r="B285" s="36" t="inlineStr">
+      <c r="B285" s="37" t="inlineStr">
         <is>
           <t>PS5-71-02 - CFO Allocation Metering Package</t>
         </is>
@@ -9003,7 +9042,7 @@
           <t>PS5-71-03</t>
         </is>
       </c>
-      <c r="B286" s="36" t="inlineStr">
+      <c r="B286" s="37" t="inlineStr">
         <is>
           <t>PS5-71-03 - CFO Allocation Metering Package (UCP)</t>
         </is>
@@ -9031,7 +9070,7 @@
           <t>PS5-71-04</t>
         </is>
       </c>
-      <c r="B287" s="36" t="inlineStr">
+      <c r="B287" s="37" t="inlineStr">
         <is>
           <t>PS5-71-04 - CFO Storage Tank</t>
         </is>
@@ -9059,7 +9098,7 @@
           <t>PS5-71-05</t>
         </is>
       </c>
-      <c r="B288" s="36" t="inlineStr">
+      <c r="B288" s="37" t="inlineStr">
         <is>
           <t>PS5-71-05 - CFO Transfer Pump A/B</t>
         </is>
@@ -9087,7 +9126,7 @@
           <t>PS5-71-06</t>
         </is>
       </c>
-      <c r="B289" s="36" t="inlineStr">
+      <c r="B289" s="37" t="inlineStr">
         <is>
           <t>PS5-71-06 - Crude Fuel Separation Module</t>
         </is>
@@ -9115,7 +9154,7 @@
           <t>PS5-71-07</t>
         </is>
       </c>
-      <c r="B290" s="36" t="inlineStr">
+      <c r="B290" s="37" t="inlineStr">
         <is>
           <t>PS5-71-07 - Crude Fuel Separation Module (UCP)</t>
         </is>
@@ -9143,7 +9182,7 @@
           <t>PS5-71-08</t>
         </is>
       </c>
-      <c r="B291" s="36" t="inlineStr">
+      <c r="B291" s="37" t="inlineStr">
         <is>
           <t>PS5-71-08 - CFO Pre-Pressure Modules</t>
         </is>
@@ -9171,7 +9210,7 @@
           <t>PS5-71-09</t>
         </is>
       </c>
-      <c r="B292" s="36" t="inlineStr">
+      <c r="B292" s="37" t="inlineStr">
         <is>
           <t>PS5-71-09 - CFO Pre-Pressure Modules (UCP)</t>
         </is>
@@ -9199,7 +9238,7 @@
           <t>PS5-71-12</t>
         </is>
       </c>
-      <c r="B293" s="36" t="inlineStr">
+      <c r="B293" s="37" t="inlineStr">
         <is>
           <t>PS5-71-12 - CFO Service Tank</t>
         </is>
@@ -9227,7 +9266,7 @@
           <t>PS5-71-13</t>
         </is>
       </c>
-      <c r="B294" s="36" t="inlineStr">
+      <c r="B294" s="37" t="inlineStr">
         <is>
           <t>PS5-71-13 - CFO Service Pump A/B</t>
         </is>
@@ -9255,7 +9294,7 @@
           <t>PS5-71-14</t>
         </is>
       </c>
-      <c r="B295" s="36" t="inlineStr">
+      <c r="B295" s="37" t="inlineStr">
         <is>
           <t>PS5-71-14 - Diesel Fuel Transfer and Dispensing Station</t>
         </is>
@@ -9283,7 +9322,7 @@
           <t>PS5-71-15</t>
         </is>
       </c>
-      <c r="B296" s="36" t="inlineStr">
+      <c r="B296" s="37" t="inlineStr">
         <is>
           <t>PS5-71-15 - Diesel Fuel Storage Tank</t>
         </is>
@@ -9311,7 +9350,7 @@
           <t>PS5-71-16</t>
         </is>
       </c>
-      <c r="B297" s="36" t="inlineStr">
+      <c r="B297" s="37" t="inlineStr">
         <is>
           <t>PS5-71-16 - Diesel Fuel Supply Pump A/B</t>
         </is>
@@ -9339,7 +9378,7 @@
           <t>PS5-71-17</t>
         </is>
       </c>
-      <c r="B298" s="36" t="inlineStr">
+      <c r="B298" s="37" t="inlineStr">
         <is>
           <t>PS5-71-17 - Diesel Fuel Distribution Header</t>
         </is>
@@ -9367,7 +9406,7 @@
           <t>PS5-71-18</t>
         </is>
       </c>
-      <c r="B299" s="36" t="inlineStr">
+      <c r="B299" s="37" t="inlineStr">
         <is>
           <t>PS5-71-18 - Diesel Separator Module</t>
         </is>
@@ -9395,7 +9434,7 @@
           <t>PS5-71-19</t>
         </is>
       </c>
-      <c r="B300" s="36" t="inlineStr">
+      <c r="B300" s="37" t="inlineStr">
         <is>
           <t>PS5-71-19 - Diesel Separator Module (UCP)</t>
         </is>
@@ -9423,7 +9462,7 @@
           <t>PS5-71-20</t>
         </is>
       </c>
-      <c r="B301" s="36" t="inlineStr">
+      <c r="B301" s="37" t="inlineStr">
         <is>
           <t>PS5-71-20 - Diesel Fuel Day Tank</t>
         </is>
@@ -9451,7 +9490,7 @@
           <t>PS5-71-21</t>
         </is>
       </c>
-      <c r="B302" s="36" t="inlineStr">
+      <c r="B302" s="37" t="inlineStr">
         <is>
           <t>PS5-71-21 - Diesel Transfer Pump A/B</t>
         </is>
@@ -9479,7 +9518,7 @@
           <t>PS5-71-22</t>
         </is>
       </c>
-      <c r="B303" s="36" t="inlineStr">
+      <c r="B303" s="37" t="inlineStr">
         <is>
           <t>PS5-71-22 - Diesel Fuel Pre Pressure Module</t>
         </is>
@@ -9507,7 +9546,7 @@
           <t>PS5-71-23</t>
         </is>
       </c>
-      <c r="B304" s="36" t="inlineStr">
+      <c r="B304" s="37" t="inlineStr">
         <is>
           <t>PS5-71-23 - Diesel Fuel Pre Pressure Module (UCP)</t>
         </is>
@@ -9535,7 +9574,7 @@
           <t>PS5-74-01</t>
         </is>
       </c>
-      <c r="B305" s="36" t="inlineStr">
+      <c r="B305" s="37" t="inlineStr">
         <is>
           <t>PS5-74-01 - N2 Generation Skid</t>
         </is>
@@ -9563,7 +9602,7 @@
           <t>PS5-74-02</t>
         </is>
       </c>
-      <c r="B306" s="36" t="inlineStr">
+      <c r="B306" s="37" t="inlineStr">
         <is>
           <t>PS5-74-02 - N2 Generation Skid (UCP)</t>
         </is>
@@ -9591,7 +9630,7 @@
           <t>PS5-74-03</t>
         </is>
       </c>
-      <c r="B307" s="36" t="inlineStr">
+      <c r="B307" s="37" t="inlineStr">
         <is>
           <t>PS5-74-03 - Nitrogen Receiver</t>
         </is>
@@ -9619,7 +9658,7 @@
           <t>PS5-74-04</t>
         </is>
       </c>
-      <c r="B308" s="36" t="inlineStr">
+      <c r="B308" s="37" t="inlineStr">
         <is>
           <t>PS5-74-04 - Nitrogen Distribution Header</t>
         </is>
@@ -9647,7 +9686,7 @@
           <t>PS5-75-01</t>
         </is>
       </c>
-      <c r="B309" s="36" t="inlineStr">
+      <c r="B309" s="37" t="inlineStr">
         <is>
           <t>PS5-75-01 - DRA Injection Package</t>
         </is>
@@ -9675,7 +9714,7 @@
           <t>PS5-75-02</t>
         </is>
       </c>
-      <c r="B310" s="36" t="inlineStr">
+      <c r="B310" s="37" t="inlineStr">
         <is>
           <t>PS5-75-02 - Biocide Injection Package</t>
         </is>
@@ -9703,7 +9742,7 @@
           <t>PS5-75-03</t>
         </is>
       </c>
-      <c r="B311" s="36" t="inlineStr">
+      <c r="B311" s="37" t="inlineStr">
         <is>
           <t>PS5-75-03 - Corrosion Inhibitor Injection Package</t>
         </is>
@@ -9731,7 +9770,7 @@
           <t>PS5-78-01</t>
         </is>
       </c>
-      <c r="B312" s="36" t="inlineStr">
+      <c r="B312" s="37" t="inlineStr">
         <is>
           <t>PS5-78-01 - Lifting and handling equipment</t>
         </is>
@@ -9759,7 +9798,7 @@
           <t>PS5-79-01</t>
         </is>
       </c>
-      <c r="B313" s="36" t="inlineStr">
+      <c r="B313" s="37" t="inlineStr">
         <is>
           <t>PS5-79-01 - Electrical Heat Tracing Transformer/Distribution Board 1 (PS5-79-IG-0001)</t>
         </is>
@@ -9787,7 +9826,7 @@
           <t>PS5-79-02</t>
         </is>
       </c>
-      <c r="B314" s="36" t="inlineStr">
+      <c r="B314" s="37" t="inlineStr">
         <is>
           <t>PS5-79-02 - Electrical Heat Tracing Transformer/Distribution Board 2 (PS5-79-IG-0002)</t>
         </is>
@@ -9815,7 +9854,7 @@
           <t>PS5-79-03</t>
         </is>
       </c>
-      <c r="B315" s="36" t="inlineStr">
+      <c r="B315" s="37" t="inlineStr">
         <is>
           <t>PS5-79-03 - Electrical Heat Tracing Transformer/Distribution Board 3 (PS5-79-IG-0003)</t>
         </is>
@@ -9843,7 +9882,7 @@
           <t>PS5-79-04</t>
         </is>
       </c>
-      <c r="B316" s="36" t="inlineStr">
+      <c r="B316" s="37" t="inlineStr">
         <is>
           <t>PS5-79-04 - Electrical Heat Tracing Transformer/Distribution Board 4 (PS5-79-IG-0004)</t>
         </is>
@@ -9871,7 +9910,7 @@
           <t>PS5-79-05</t>
         </is>
       </c>
-      <c r="B317" s="36" t="inlineStr">
+      <c r="B317" s="37" t="inlineStr">
         <is>
           <t>PS5-79-05 - Electrical Heat Tracing Transformer/Distribution Board 5 (PS5-79-IG-0005)</t>
         </is>
@@ -9899,7 +9938,7 @@
           <t>PS5-79-06</t>
         </is>
       </c>
-      <c r="B318" s="36" t="inlineStr">
+      <c r="B318" s="37" t="inlineStr">
         <is>
           <t>PS5-79-06 - Electrical Heat Tracing Transformer/Distribution Board 6 (PS5-79-IG-0006)</t>
         </is>
@@ -9927,7 +9966,7 @@
           <t>PS5-79-07</t>
         </is>
       </c>
-      <c r="B319" s="36" t="inlineStr">
+      <c r="B319" s="37" t="inlineStr">
         <is>
           <t>PS5-79-07 - Electrical Heat Tracing Transformer/Distribution Board 7 (PS5-79-IG-0007)</t>
         </is>
@@ -9955,7 +9994,7 @@
           <t>PS5-79-08</t>
         </is>
       </c>
-      <c r="B320" s="36" t="inlineStr">
+      <c r="B320" s="37" t="inlineStr">
         <is>
           <t>PS5-79-08 - Electrical Heat Tracing Transformer/Distribution Board 8 (PS5-79-IG-0008)</t>
         </is>
@@ -9983,7 +10022,7 @@
           <t>PS5-79-09</t>
         </is>
       </c>
-      <c r="B321" s="36" t="inlineStr">
+      <c r="B321" s="37" t="inlineStr">
         <is>
           <t>PS5-79-09 - Electrical Heat Tracing Transformer/Distribution Board 9 (PS5-79-IG-0009)</t>
         </is>
@@ -10011,7 +10050,7 @@
           <t>PS5-79-10</t>
         </is>
       </c>
-      <c r="B322" s="36" t="inlineStr">
+      <c r="B322" s="37" t="inlineStr">
         <is>
           <t>PS5-79-10 - Electrical Heat Tracing Transformer/Distribution Board 10 (PS5-79-IG-0010)</t>
         </is>
@@ -10039,7 +10078,7 @@
           <t>PS5-79-11</t>
         </is>
       </c>
-      <c r="B323" s="36" t="inlineStr">
+      <c r="B323" s="37" t="inlineStr">
         <is>
           <t>PS5-79-11 - Electrical Heat Tracing Transformer/Distribution Board 11 (PS5-79-IG-0011)</t>
         </is>
@@ -10067,7 +10106,7 @@
           <t>PS5-79-12</t>
         </is>
       </c>
-      <c r="B324" s="36" t="inlineStr">
+      <c r="B324" s="37" t="inlineStr">
         <is>
           <t>PS5-79-12 - Electrical Heat Tracing Transformer/Distribution Board 12 (PS5-79-IG-0012)</t>
         </is>
@@ -10095,7 +10134,7 @@
           <t>PS5-82-01</t>
         </is>
       </c>
-      <c r="B325" s="36" t="inlineStr">
+      <c r="B325" s="37" t="inlineStr">
         <is>
           <t>PS5-82-01 - Sanitary Sewage Collection</t>
         </is>
@@ -10123,7 +10162,7 @@
           <t>PS5-82-02</t>
         </is>
       </c>
-      <c r="B326" s="36" t="inlineStr">
+      <c r="B326" s="37" t="inlineStr">
         <is>
           <t>PS5-82-02 - Sewage Treatment Plant Package</t>
         </is>
@@ -10151,7 +10190,7 @@
           <t>PS5-82-03</t>
         </is>
       </c>
-      <c r="B327" s="36" t="inlineStr">
+      <c r="B327" s="37" t="inlineStr">
         <is>
           <t>PS5-82-03 - Sewage Treatment Plant Package (UCP)</t>
         </is>
@@ -10179,7 +10218,7 @@
           <t>PS5-82-04</t>
         </is>
       </c>
-      <c r="B328" s="36" t="inlineStr">
+      <c r="B328" s="37" t="inlineStr">
         <is>
           <t>PS5-82-04 - Sewage Treatment Plant Discharge Piping</t>
         </is>
@@ -10207,7 +10246,7 @@
           <t>PS5-82-05</t>
         </is>
       </c>
-      <c r="B329" s="36" t="inlineStr">
+      <c r="B329" s="37" t="inlineStr">
         <is>
           <t>PS5-82-05 - Office and Facilities building</t>
         </is>
@@ -10235,7 +10274,7 @@
           <t>PS5-82-06</t>
         </is>
       </c>
-      <c r="B330" s="36" t="inlineStr">
+      <c r="B330" s="37" t="inlineStr">
         <is>
           <t>PS5-82-06 - Guard House Building</t>
         </is>
@@ -10263,7 +10302,7 @@
           <t>PS5-82-07</t>
         </is>
       </c>
-      <c r="B331" s="36" t="inlineStr">
+      <c r="B331" s="37" t="inlineStr">
         <is>
           <t>PS5-82-07 - Guard Huts</t>
         </is>
@@ -10291,7 +10330,7 @@
           <t>PS5-83-01</t>
         </is>
       </c>
-      <c r="B332" s="36" t="inlineStr">
+      <c r="B332" s="37" t="inlineStr">
         <is>
           <t>PS5-83-01 - EITS Building</t>
         </is>
@@ -10319,7 +10358,7 @@
           <t>PS5-84-01</t>
         </is>
       </c>
-      <c r="B333" s="36" t="inlineStr">
+      <c r="B333" s="37" t="inlineStr">
         <is>
           <t>PS5-84-01 - Generator Building</t>
         </is>
@@ -10347,7 +10386,7 @@
           <t>PS5-84-02</t>
         </is>
       </c>
-      <c r="B334" s="36" t="inlineStr">
+      <c r="B334" s="37" t="inlineStr">
         <is>
           <t>PS5-84-02 - Workshop &amp; Warehouse</t>
         </is>
@@ -10375,7 +10414,7 @@
           <t>PS5-84-03</t>
         </is>
       </c>
-      <c r="B335" s="36" t="inlineStr">
+      <c r="B335" s="37" t="inlineStr">
         <is>
           <t>PS5-84-03 - Shelters</t>
         </is>
@@ -10403,7 +10442,7 @@
           <t>PS5-86-01</t>
         </is>
       </c>
-      <c r="B336" s="36" t="inlineStr">
+      <c r="B336" s="37" t="inlineStr">
         <is>
           <t>PS5-86-01 - Shelters</t>
         </is>
@@ -10431,7 +10470,7 @@
           <t>PS5-91-01</t>
         </is>
       </c>
-      <c r="B337" s="36" t="inlineStr">
+      <c r="B337" s="37" t="inlineStr">
         <is>
           <t>PS5-91-01 - Multicore cables &amp; JB</t>
         </is>
@@ -10459,7 +10498,7 @@
           <t>PS5-99-01</t>
         </is>
       </c>
-      <c r="B338" s="36" t="inlineStr">
+      <c r="B338" s="37" t="inlineStr">
         <is>
           <t>PS5-99-01 - Area Completion for Building area</t>
         </is>
@@ -10487,7 +10526,7 @@
           <t>PS5-99-02</t>
         </is>
       </c>
-      <c r="B339" s="36" t="inlineStr">
+      <c r="B339" s="37" t="inlineStr">
         <is>
           <t>PS5-99-02 - Area Completion for Utility area</t>
         </is>
@@ -10515,7 +10554,7 @@
           <t>PS5-99-03</t>
         </is>
       </c>
-      <c r="B340" s="36" t="inlineStr">
+      <c r="B340" s="37" t="inlineStr">
         <is>
           <t>PS5-99-03 - Area Completion for Power Distribution area</t>
         </is>
@@ -10543,7 +10582,7 @@
           <t>PS5-99-04</t>
         </is>
       </c>
-      <c r="B341" s="36" t="inlineStr">
+      <c r="B341" s="37" t="inlineStr">
         <is>
           <t>PS5-99-04 - Area Completion for Process area</t>
         </is>
@@ -10571,7 +10610,7 @@
           <t>PS5-99-05</t>
         </is>
       </c>
-      <c r="B342" s="36" t="inlineStr">
+      <c r="B342" s="37" t="inlineStr">
         <is>
           <t>PS5-99-05 - Area Completion for CFO area</t>
         </is>
@@ -10599,7 +10638,7 @@
           <t>PS5-99-06</t>
         </is>
       </c>
-      <c r="B343" s="36" t="inlineStr">
+      <c r="B343" s="37" t="inlineStr">
         <is>
           <t>PS5-99-06 - Area Completion for Power Generation area</t>
         </is>

</xml_diff>

<commit_message>
Auto sync build outputs after stash rebase
</commit_message>
<xml_diff>
--- a/EXCEL/1 - DASHBOARD.xlsx
+++ b/EXCEL/1 - DASHBOARD.xlsx
@@ -239,12 +239,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFffeb9c"/>
-        <bgColor rgb="FFffeb9c"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFe8d5c4"/>
         <bgColor rgb="FFe8d5c4"/>
       </patternFill>
@@ -313,6 +307,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFBDD7EE"/>
         <bgColor rgb="FFBDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFffeb9c"/>
+        <bgColor rgb="FFffeb9c"/>
       </patternFill>
     </fill>
     <fill>
@@ -574,7 +574,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="21" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="35" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -642,10 +642,13 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -669,25 +672,22 @@
     <xf numFmtId="0" fontId="6" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="22" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -696,13 +696,13 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="27" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -720,10 +720,10 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="28" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -738,7 +738,7 @@
     <xf numFmtId="0" fontId="4" fillId="29" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -771,16 +771,16 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1183,14 +1183,14 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="8" t="n">
-        <v>23537</v>
+        <v>23477</v>
       </c>
       <c r="B2" s="9" t="n">
-        <v>10354</v>
+        <v>12308</v>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>44%</t>
+          <t>52%</t>
         </is>
       </c>
       <c r="D2" s="11" t="n">
@@ -1206,7 +1206,7 @@
         <v>290</v>
       </c>
       <c r="H2" s="9" t="n">
-        <v>36</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
@@ -1384,18 +1384,18 @@
         </is>
       </c>
       <c r="C9" s="23" t="n">
-        <v>2405</v>
+        <v>2404</v>
       </c>
       <c r="D9" s="23" t="n">
-        <v>980</v>
+        <v>1130</v>
       </c>
       <c r="E9" s="25" t="inlineStr">
         <is>
-          <t>41%</t>
+          <t>47%</t>
         </is>
       </c>
       <c r="F9" s="23" t="n">
-        <v>1425</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="10">
@@ -1413,15 +1413,15 @@
         <v>197</v>
       </c>
       <c r="D10" s="23" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="E10" s="25" t="inlineStr">
         <is>
-          <t>36%</t>
+          <t>40%</t>
         </is>
       </c>
       <c r="F10" s="23" t="n">
-        <v>127</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11">
@@ -1436,18 +1436,18 @@
         </is>
       </c>
       <c r="C11" s="23" t="n">
-        <v>4689</v>
+        <v>4690</v>
       </c>
       <c r="D11" s="23" t="n">
-        <v>1917</v>
-      </c>
-      <c r="E11" s="25" t="inlineStr">
-        <is>
-          <t>41%</t>
+        <v>2504</v>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>53%</t>
         </is>
       </c>
       <c r="F11" s="23" t="n">
-        <v>2772</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="12">
@@ -1462,18 +1462,18 @@
         </is>
       </c>
       <c r="C12" s="23" t="n">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D12" s="23" t="n">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="E12" s="25" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>45%</t>
         </is>
       </c>
       <c r="F12" s="23" t="n">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="13">
@@ -1488,18 +1488,18 @@
         </is>
       </c>
       <c r="C13" s="23" t="n">
-        <v>1530</v>
+        <v>1477</v>
       </c>
       <c r="D13" s="23" t="n">
-        <v>1116</v>
+        <v>1272</v>
       </c>
       <c r="E13" s="26" t="inlineStr">
         <is>
-          <t>73%</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="F13" s="23" t="n">
-        <v>414</v>
+        <v>205</v>
       </c>
     </row>
     <row r="14">
@@ -1517,15 +1517,15 @@
         <v>180</v>
       </c>
       <c r="D14" s="23" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E14" s="25" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>12%</t>
         </is>
       </c>
       <c r="F14" s="23" t="n">
-        <v>172</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15">
@@ -1543,15 +1543,15 @@
         <v>3021</v>
       </c>
       <c r="D15" s="23" t="n">
-        <v>484</v>
+        <v>580</v>
       </c>
       <c r="E15" s="25" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>19%</t>
         </is>
       </c>
       <c r="F15" s="23" t="n">
-        <v>2537</v>
+        <v>2441</v>
       </c>
     </row>
     <row r="16">
@@ -1566,18 +1566,18 @@
         </is>
       </c>
       <c r="C16" s="27" t="n">
-        <v>12285</v>
+        <v>12233</v>
       </c>
       <c r="D16" s="27" t="n">
-        <v>4689</v>
+        <v>5705</v>
       </c>
       <c r="E16" s="25" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>47%</t>
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>7596</v>
+        <v>6528</v>
       </c>
     </row>
     <row r="17">
@@ -1618,18 +1618,18 @@
         </is>
       </c>
       <c r="C18" s="23" t="n">
-        <v>5889</v>
+        <v>5895</v>
       </c>
       <c r="D18" s="23" t="n">
-        <v>2186</v>
+        <v>2691</v>
       </c>
       <c r="E18" s="25" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>46%</t>
         </is>
       </c>
       <c r="F18" s="23" t="n">
-        <v>3703</v>
+        <v>3204</v>
       </c>
     </row>
     <row r="19">
@@ -1670,18 +1670,18 @@
         </is>
       </c>
       <c r="C20" s="23" t="n">
-        <v>2456</v>
+        <v>2461</v>
       </c>
       <c r="D20" s="23" t="n">
-        <v>1409</v>
+        <v>1692</v>
       </c>
       <c r="E20" s="26" t="inlineStr">
         <is>
-          <t>57%</t>
+          <t>69%</t>
         </is>
       </c>
       <c r="F20" s="23" t="n">
-        <v>1047</v>
+        <v>769</v>
       </c>
     </row>
     <row r="21">
@@ -1699,15 +1699,15 @@
         <v>553</v>
       </c>
       <c r="D21" s="23" t="n">
-        <v>304</v>
+        <v>319</v>
       </c>
       <c r="E21" s="26" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>58%</t>
         </is>
       </c>
       <c r="F21" s="23" t="n">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="22">
@@ -1722,18 +1722,18 @@
         </is>
       </c>
       <c r="C22" s="23" t="n">
-        <v>1656</v>
+        <v>1637</v>
       </c>
       <c r="D22" s="23" t="n">
-        <v>1351</v>
+        <v>1463</v>
       </c>
       <c r="E22" s="26" t="inlineStr">
         <is>
-          <t>82%</t>
+          <t>89%</t>
         </is>
       </c>
       <c r="F22" s="23" t="n">
-        <v>305</v>
+        <v>174</v>
       </c>
     </row>
     <row r="23">
@@ -1777,15 +1777,15 @@
         <v>272</v>
       </c>
       <c r="D24" s="23" t="n">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="E24" s="26" t="inlineStr">
         <is>
-          <t>56%</t>
+          <t>58%</t>
         </is>
       </c>
       <c r="F24" s="23" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="25">
@@ -1800,18 +1800,18 @@
         </is>
       </c>
       <c r="C25" s="27" t="n">
-        <v>10826</v>
+        <v>10818</v>
       </c>
       <c r="D25" s="27" t="n">
-        <v>5402</v>
+        <v>6323</v>
       </c>
       <c r="E25" s="26" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>58%</t>
         </is>
       </c>
       <c r="F25" s="27" t="n">
-        <v>5424</v>
+        <v>4495</v>
       </c>
     </row>
     <row r="26">
@@ -1829,15 +1829,15 @@
         <v>74</v>
       </c>
       <c r="D26" s="23" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E26" s="25" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="F26" s="23" t="n">
-        <v>63</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27">
@@ -1855,15 +1855,15 @@
         <v>34</v>
       </c>
       <c r="D27" s="23" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E27" s="25" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="F27" s="23" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="28">
@@ -1907,7 +1907,7 @@
         <v>200</v>
       </c>
       <c r="D29" s="23" t="n">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E29" s="29" t="inlineStr">
         <is>
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="F29" s="23" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="30">
@@ -1933,15 +1933,15 @@
         <v>23</v>
       </c>
       <c r="D30" s="23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E30" s="25" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="F30" s="23" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="31">
@@ -1959,15 +1959,15 @@
         <v>66</v>
       </c>
       <c r="D31" s="23" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E31" s="26" t="inlineStr">
         <is>
-          <t>53%</t>
+          <t>55%</t>
         </is>
       </c>
       <c r="F31" s="23" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32">
@@ -2037,15 +2037,15 @@
         <v>397</v>
       </c>
       <c r="D34" s="27" t="n">
-        <v>243</v>
+        <v>260</v>
       </c>
       <c r="E34" s="26" t="inlineStr">
         <is>
-          <t>61%</t>
+          <t>65%</t>
         </is>
       </c>
       <c r="F34" s="27" t="n">
-        <v>154</v>
+        <v>137</v>
       </c>
     </row>
     <row r="35">
@@ -2060,18 +2060,18 @@
         </is>
       </c>
       <c r="C35" s="30" t="n">
-        <v>15480</v>
+        <v>15509</v>
       </c>
       <c r="D35" s="30" t="n">
-        <v>8254</v>
+        <v>9856</v>
       </c>
       <c r="E35" s="26" t="inlineStr">
         <is>
-          <t>53%</t>
+          <t>64%</t>
         </is>
       </c>
       <c r="F35" s="30" t="n">
-        <v>7226</v>
+        <v>5653</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">

</xml_diff>

<commit_message>
Full sync: platform + all Excel downloads
</commit_message>
<xml_diff>
--- a/EXCEL/1 - DASHBOARD.xlsx
+++ b/EXCEL/1 - DASHBOARD.xlsx
@@ -1183,14 +1183,14 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="8" t="n">
-        <v>23477</v>
+        <v>23483</v>
       </c>
       <c r="B2" s="9" t="n">
-        <v>12308</v>
+        <v>12875</v>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>55%</t>
         </is>
       </c>
       <c r="D2" s="11" t="n">
@@ -1206,7 +1206,7 @@
         <v>290</v>
       </c>
       <c r="H2" s="9" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
@@ -1384,18 +1384,18 @@
         </is>
       </c>
       <c r="C9" s="23" t="n">
-        <v>2404</v>
+        <v>2403</v>
       </c>
       <c r="D9" s="23" t="n">
-        <v>1130</v>
+        <v>1152</v>
       </c>
       <c r="E9" s="25" t="inlineStr">
         <is>
-          <t>47%</t>
+          <t>48%</t>
         </is>
       </c>
       <c r="F9" s="23" t="n">
-        <v>1274</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="10">
@@ -1439,15 +1439,15 @@
         <v>4690</v>
       </c>
       <c r="D11" s="23" t="n">
-        <v>2504</v>
+        <v>2617</v>
       </c>
       <c r="E11" s="26" t="inlineStr">
         <is>
-          <t>53%</t>
+          <t>56%</t>
         </is>
       </c>
       <c r="F11" s="23" t="n">
-        <v>2186</v>
+        <v>2073</v>
       </c>
     </row>
     <row r="12">
@@ -1488,18 +1488,18 @@
         </is>
       </c>
       <c r="C13" s="23" t="n">
-        <v>1477</v>
+        <v>1478</v>
       </c>
       <c r="D13" s="23" t="n">
-        <v>1272</v>
+        <v>1291</v>
       </c>
       <c r="E13" s="26" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="F13" s="23" t="n">
-        <v>205</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14">
@@ -1517,15 +1517,15 @@
         <v>180</v>
       </c>
       <c r="D14" s="23" t="n">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="E14" s="25" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>21%</t>
         </is>
       </c>
       <c r="F14" s="23" t="n">
-        <v>158</v>
+        <v>143</v>
       </c>
     </row>
     <row r="15">
@@ -1543,15 +1543,15 @@
         <v>3021</v>
       </c>
       <c r="D15" s="23" t="n">
-        <v>580</v>
+        <v>603</v>
       </c>
       <c r="E15" s="25" t="inlineStr">
         <is>
-          <t>19%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="F15" s="23" t="n">
-        <v>2441</v>
+        <v>2418</v>
       </c>
     </row>
     <row r="16">
@@ -1569,15 +1569,15 @@
         <v>12233</v>
       </c>
       <c r="D16" s="27" t="n">
-        <v>5705</v>
+        <v>5897</v>
       </c>
       <c r="E16" s="25" t="inlineStr">
         <is>
-          <t>47%</t>
+          <t>48%</t>
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>6528</v>
+        <v>6336</v>
       </c>
     </row>
     <row r="17">
@@ -1618,18 +1618,18 @@
         </is>
       </c>
       <c r="C18" s="23" t="n">
-        <v>5895</v>
+        <v>5896</v>
       </c>
       <c r="D18" s="23" t="n">
-        <v>2691</v>
+        <v>2900</v>
       </c>
       <c r="E18" s="25" t="inlineStr">
         <is>
-          <t>46%</t>
+          <t>49%</t>
         </is>
       </c>
       <c r="F18" s="23" t="n">
-        <v>3204</v>
+        <v>2996</v>
       </c>
     </row>
     <row r="19">
@@ -1670,18 +1670,18 @@
         </is>
       </c>
       <c r="C20" s="23" t="n">
-        <v>2461</v>
+        <v>2462</v>
       </c>
       <c r="D20" s="23" t="n">
-        <v>1692</v>
+        <v>1785</v>
       </c>
       <c r="E20" s="26" t="inlineStr">
         <is>
-          <t>69%</t>
+          <t>73%</t>
         </is>
       </c>
       <c r="F20" s="23" t="n">
-        <v>769</v>
+        <v>677</v>
       </c>
     </row>
     <row r="21">
@@ -1696,18 +1696,18 @@
         </is>
       </c>
       <c r="C21" s="23" t="n">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="D21" s="23" t="n">
-        <v>319</v>
+        <v>339</v>
       </c>
       <c r="E21" s="26" t="inlineStr">
         <is>
-          <t>58%</t>
+          <t>61%</t>
         </is>
       </c>
       <c r="F21" s="23" t="n">
-        <v>234</v>
+        <v>215</v>
       </c>
     </row>
     <row r="22">
@@ -1722,18 +1722,18 @@
         </is>
       </c>
       <c r="C22" s="23" t="n">
-        <v>1637</v>
+        <v>1641</v>
       </c>
       <c r="D22" s="23" t="n">
-        <v>1463</v>
-      </c>
-      <c r="E22" s="26" t="inlineStr">
-        <is>
-          <t>89%</t>
+        <v>1485</v>
+      </c>
+      <c r="E22" s="29" t="inlineStr">
+        <is>
+          <t>90%</t>
         </is>
       </c>
       <c r="F22" s="23" t="n">
-        <v>174</v>
+        <v>156</v>
       </c>
     </row>
     <row r="23">
@@ -1777,15 +1777,15 @@
         <v>272</v>
       </c>
       <c r="D24" s="23" t="n">
-        <v>158</v>
+        <v>188</v>
       </c>
       <c r="E24" s="26" t="inlineStr">
         <is>
-          <t>58%</t>
+          <t>69%</t>
         </is>
       </c>
       <c r="F24" s="23" t="n">
-        <v>114</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25">
@@ -1800,18 +1800,18 @@
         </is>
       </c>
       <c r="C25" s="27" t="n">
-        <v>10818</v>
+        <v>10825</v>
       </c>
       <c r="D25" s="27" t="n">
-        <v>6323</v>
+        <v>6697</v>
       </c>
       <c r="E25" s="26" t="inlineStr">
         <is>
-          <t>58%</t>
+          <t>62%</t>
         </is>
       </c>
       <c r="F25" s="27" t="n">
-        <v>4495</v>
+        <v>4128</v>
       </c>
     </row>
     <row r="26">
@@ -1826,18 +1826,18 @@
         </is>
       </c>
       <c r="C26" s="23" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D26" s="23" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E26" s="25" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="F26" s="23" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27">
@@ -2034,18 +2034,18 @@
         </is>
       </c>
       <c r="C34" s="27" t="n">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="D34" s="27" t="n">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E34" s="26" t="inlineStr">
         <is>
-          <t>65%</t>
+          <t>66%</t>
         </is>
       </c>
       <c r="F34" s="27" t="n">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="35">
@@ -2060,18 +2060,18 @@
         </is>
       </c>
       <c r="C35" s="30" t="n">
-        <v>15509</v>
+        <v>15512</v>
       </c>
       <c r="D35" s="30" t="n">
-        <v>9856</v>
+        <v>10195</v>
       </c>
       <c r="E35" s="26" t="inlineStr">
         <is>
-          <t>64%</t>
+          <t>66%</t>
         </is>
       </c>
       <c r="F35" s="30" t="n">
-        <v>5653</v>
+        <v>5317</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">

</xml_diff>